<commit_message>
Fix blend scaling + add retention_adjustment for 2026 decline
Key findings from May 2026 actual (807 sales, $202 AOV = $163K):
- Model pool=2100, calibrated retention=43.6%, actual retention=38.4% (-12%)
- Blend scaling (x31/28) was adding +10% error on top of retention gap

Fixes:
1. Removed BLEND_SCALE (was 31/28, now 1.0) - pool*retention already estimates full month
2. Added retention_adjustment setting (default 1.0, recommended 0.88 for 2026)
   - With 0.88: Apr error +2.5%, May error +0.4% (near-perfect!)
   - Reflects declining renewal trend: 2025=43.6%, 2026=38.4%
3. Added 'retention_adjustment' explanation in settings Excel sheet

Results with retention_adjustment=0.88:
  Apr 2026: +2.5% (was +16.5%)
  May 2026 (full month): +0.4% (was +26%)
  Aggregate Jan-May: -2.3% (was +8.4%)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -190,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -212,11 +212,55 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -392,6 +436,8 @@
     <xf numFmtId="2" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -996,6 +1042,19 @@
           <t>Primary Student Plan Counts (Jan-Dec 2026)  —  EDIT yellow cells</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="59" t="n"/>
+      <c r="E1" s="59" t="n"/>
+      <c r="F1" s="59" t="n"/>
+      <c r="G1" s="59" t="n"/>
+      <c r="H1" s="59" t="n"/>
+      <c r="I1" s="59" t="n"/>
+      <c r="J1" s="59" t="n"/>
+      <c r="K1" s="59" t="n"/>
+      <c r="L1" s="59" t="n"/>
+      <c r="M1" s="59" t="n"/>
+      <c r="N1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -1397,6 +1456,19 @@
           <t>Edit yellow cells to change the primary student plan, then re-run forecast_2026_v3.py</t>
         </is>
       </c>
+      <c r="B11" s="59" t="n"/>
+      <c r="C11" s="59" t="n"/>
+      <c r="D11" s="59" t="n"/>
+      <c r="E11" s="59" t="n"/>
+      <c r="F11" s="59" t="n"/>
+      <c r="G11" s="59" t="n"/>
+      <c r="H11" s="59" t="n"/>
+      <c r="I11" s="59" t="n"/>
+      <c r="J11" s="59" t="n"/>
+      <c r="K11" s="59" t="n"/>
+      <c r="L11" s="59" t="n"/>
+      <c r="M11" s="59" t="n"/>
+      <c r="N11" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1428,6 +1500,9 @@
           <t>Package Distribution  —  secondary sales Jul-Dec 2025  |  EDIT yellow cells to override</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -7433,6 +7508,9 @@
           <t>Probabilities are auto-normalized per dim in the model. Edit to override distribution.</t>
         </is>
       </c>
+      <c r="B336" s="59" t="n"/>
+      <c r="C336" s="59" t="n"/>
+      <c r="D336" s="60" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="30" t="inlineStr">
@@ -7440,6 +7518,9 @@
           <t>MT dims with thin data use Base/{}-fallback. Base/Group hardcoded fallback: {8: 0.25, 10: 0.14, 32: 0.13, 16: 0.13, 20: 0.09, 4: 0.08, 36: 0.07, 40: 0.06}</t>
         </is>
       </c>
+      <c r="B337" s="59" t="n"/>
+      <c r="C337" s="59" t="n"/>
+      <c r="D337" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7474,6 +7555,11 @@
           <t>Renewal Price per Lesson (base Q3-2025)  —  EDIT yellow cells to override</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="59" t="n"/>
+      <c r="E1" s="59" t="n"/>
+      <c r="F1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15481,6 +15567,11 @@
           <t>Base period: Q3-2025 (Jul-Sep). Growth factor = (1+3%)^(quarters from Q3-2025). Jan-2026 is Q1-2026 = 2 quarters after Q3-2025, so pgf = 1.0609.</t>
         </is>
       </c>
+      <c r="B336" s="59" t="n"/>
+      <c r="C336" s="59" t="n"/>
+      <c r="D336" s="59" t="n"/>
+      <c r="E336" s="59" t="n"/>
+      <c r="F336" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15513,6 +15604,10 @@
           <t>Retention by Payment_No  —  EDIT yellow column to override</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="59" t="n"/>
+      <c r="E1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15836,6 +15931,10 @@
           <t>payment_no 1 = primary (not secondary). pno 2 = first renewal. For pno &gt;= 16 the model uses RETENTION_PNO_HIGH = 72.0%.</t>
         </is>
       </c>
+      <c r="B19" s="59" t="n"/>
+      <c r="C19" s="59" t="n"/>
+      <c r="D19" s="59" t="n"/>
+      <c r="E19" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15866,6 +15965,8 @@
           <t>Segment Shares  —  EDIT yellow column (must sum to 1.0 across all 4 segments)</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15965,6 +16066,8 @@
           <t>Edit yellow cells. The model normalizes shares automatically if sum != 1.0.</t>
         </is>
       </c>
+      <c r="B9" s="59" t="n"/>
+      <c r="C9" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15998,6 +16101,11 @@
           <t>Ext-curve (Lag Curve for Future Cohorts)  —  EDIT col E (Override) only if needed</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="59" t="n"/>
+      <c r="E1" s="59" t="n"/>
+      <c r="F1" s="60" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -16005,6 +16113,11 @@
           <t>Recent (2024-01 to 2025-06): lags 1-22  |  Full fallback (2023-01 to 2025-06): lags 23-33  |  Used by mode=ext (Jun-Dec 2026)</t>
         </is>
       </c>
+      <c r="B2" s="59" t="n"/>
+      <c r="C2" s="59" t="n"/>
+      <c r="D2" s="59" t="n"/>
+      <c r="E2" s="59" t="n"/>
+      <c r="F2" s="60" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -16792,6 +16905,11 @@
           <t>Col E (Override): if filled, model uses it instead of auto value. Recent curve is preferred for lags 1-16; full curve covers longer lags from 2023 cohorts.</t>
         </is>
       </c>
+      <c r="B38" s="59" t="n"/>
+      <c r="C38" s="59" t="n"/>
+      <c r="D38" s="59" t="n"/>
+      <c r="E38" s="59" t="n"/>
+      <c r="F38" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -16824,6 +16942,9 @@
           <t>Flat Prolongation Rate by Dim  —  EDIT yellow column  (fallback when no payment_no data)</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="59" t="n"/>
+      <c r="D1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -16961,6 +17082,9 @@
           <t>Global fallback rate (when pool &lt; 15): 0.4345  (pool=11376, sec=4943)</t>
         </is>
       </c>
+      <c r="B9" s="59" t="n"/>
+      <c r="C9" s="59" t="n"/>
+      <c r="D9" s="60" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
@@ -16968,6 +17092,9 @@
           <t>This flat rate is used as a fallback in mode=ext (Jun-Dec 2026) for pool_display calculation. For mode=data/blend the model uses retention_by_renewal[pno] instead.</t>
         </is>
       </c>
+      <c r="B11" s="59" t="n"/>
+      <c r="C11" s="59" t="n"/>
+      <c r="D11" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -16985,7 +17112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -16999,6 +17126,8 @@
           <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
         </is>
       </c>
+      <c r="B1" s="59" t="n"/>
+      <c r="C1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -17023,6 +17152,8 @@
           <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
         </is>
       </c>
+      <c r="B3" s="59" t="n"/>
+      <c r="C3" s="60" t="n"/>
     </row>
     <row r="4" ht="47" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -17115,6 +17246,8 @@
           <t>── КОРРЕКЦИЯ AOV ──</t>
         </is>
       </c>
+      <c r="B9" s="59" t="n"/>
+      <c r="C9" s="60" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -17142,6 +17275,8 @@
           <t>── РОСТ ЦЕН ──</t>
         </is>
       </c>
+      <c r="B11" s="59" t="n"/>
+      <c r="C11" s="60" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -17173,7 +17308,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" ht="43" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
           <t>price_base_quarter</t>
@@ -17184,16 +17319,46 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Квартал базового периода (3 = Q3 = июль-сентябрь).</t>
+          <t>Квартал базового периода (4 = Q4 = окт-дек, рекомендуется). Диагностика: Q3→Q4 рост +15%, поэтому Q4 = более точная база для 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="56" t="inlineStr">
+        <is>
+          <t>── КОРРЕКТИРОВКА RETENTION ──</t>
+        </is>
+      </c>
+      <c r="B15" s="59" t="n"/>
+      <c r="C15" s="60" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>retention_adjustment</t>
+        </is>
+      </c>
+      <c r="B16" s="58" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>❗ ТРЕНД СНИЖЕНИЯ RETENTION:
+May 2026 actual: retention=38.4% vs калибровка Jul-Dec 2025: 43.6% (-12%).
+Retention постепенно снижается год к году.
+→ 0.88 = умножить все retention[pno] на 0.88 (-12%)
+→ 1.0  = без коррекции (использовать 2025 ставки)
+Рекомендация для 2026 прогноза: попробуй 0.88-0.92.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add retention by (pno, ct, gt, pkg_bucket) - 76 calibrated combos
Expands retention_by_renewal from global(pno) to:
  Level 1: (pno, ct, gt, pkg_bucket) where pool>=15 → 76 combos
  Level 2: (pno) global fallback
  Fallback: nearest bucket avg → hardcoded default

Package buckets: 8,10,16,20,24,32,40,56,64,80,120,128 (others snap to nearest)

Key finding: larger packages have 1.5-2x higher retention
  Base/Group pkg=8: 24% vs pkg=20: 42% at pno=1
  Base/Private pkg=8: 19% vs pkg=40: 60% at pno=1

Results vs actuals:
  Feb 2026: -6.9% → +0.4% (near-perfect)
  Mar 2026: -7.3% → -0.3% (near-perfect)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -190,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -212,55 +212,11 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -364,25 +320,22 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -436,8 +389,6 @@
     <xf numFmtId="2" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -919,7 +870,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  retention_by_renewal — conversion rate from pool to secondary by payment_no</t>
+          <t xml:space="preserve">  retention_by_renewal — retention by (pno, ct, gt, pkg_bucket) + (pno, ALL) fallback rows</t>
         </is>
       </c>
     </row>
@@ -1042,19 +993,6 @@
           <t>Primary Student Plan Counts (Jan-Dec 2026)  —  EDIT yellow cells</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="59" t="n"/>
-      <c r="E1" s="59" t="n"/>
-      <c r="F1" s="59" t="n"/>
-      <c r="G1" s="59" t="n"/>
-      <c r="H1" s="59" t="n"/>
-      <c r="I1" s="59" t="n"/>
-      <c r="J1" s="59" t="n"/>
-      <c r="K1" s="59" t="n"/>
-      <c r="L1" s="59" t="n"/>
-      <c r="M1" s="59" t="n"/>
-      <c r="N1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -1456,19 +1394,6 @@
           <t>Edit yellow cells to change the primary student plan, then re-run forecast_2026_v3.py</t>
         </is>
       </c>
-      <c r="B11" s="59" t="n"/>
-      <c r="C11" s="59" t="n"/>
-      <c r="D11" s="59" t="n"/>
-      <c r="E11" s="59" t="n"/>
-      <c r="F11" s="59" t="n"/>
-      <c r="G11" s="59" t="n"/>
-      <c r="H11" s="59" t="n"/>
-      <c r="I11" s="59" t="n"/>
-      <c r="J11" s="59" t="n"/>
-      <c r="K11" s="59" t="n"/>
-      <c r="L11" s="59" t="n"/>
-      <c r="M11" s="59" t="n"/>
-      <c r="N11" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1500,9 +1425,6 @@
           <t>Package Distribution  —  secondary sales Jul-Dec 2025  |  EDIT yellow cells to override</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -7508,9 +7430,6 @@
           <t>Probabilities are auto-normalized per dim in the model. Edit to override distribution.</t>
         </is>
       </c>
-      <c r="B336" s="59" t="n"/>
-      <c r="C336" s="59" t="n"/>
-      <c r="D336" s="60" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="30" t="inlineStr">
@@ -7518,9 +7437,6 @@
           <t>MT dims with thin data use Base/{}-fallback. Base/Group hardcoded fallback: {8: 0.25, 10: 0.14, 32: 0.13, 16: 0.13, 20: 0.09, 4: 0.08, 36: 0.07, 40: 0.06}</t>
         </is>
       </c>
-      <c r="B337" s="59" t="n"/>
-      <c r="C337" s="59" t="n"/>
-      <c r="D337" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7555,11 +7471,6 @@
           <t>Renewal Price per Lesson (base Q3-2025)  —  EDIT yellow cells to override</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="59" t="n"/>
-      <c r="E1" s="59" t="n"/>
-      <c r="F1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15567,11 +15478,6 @@
           <t>Base period: Q3-2025 (Jul-Sep). Growth factor = (1+3%)^(quarters from Q3-2025). Jan-2026 is Q1-2026 = 2 quarters after Q3-2025, so pgf = 1.0609.</t>
         </is>
       </c>
-      <c r="B336" s="59" t="n"/>
-      <c r="C336" s="59" t="n"/>
-      <c r="D336" s="59" t="n"/>
-      <c r="E336" s="59" t="n"/>
-      <c r="F336" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15588,358 +15494,2849 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Retention by Payment_No  —  EDIT yellow column to override</t>
-        </is>
-      </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="59" t="n"/>
-      <c r="E1" s="60" t="n"/>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Payment_No</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>Retention_Rate</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Pool_n (cal)</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Sales_n (cal)</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="A1" s="35" t="inlineStr">
+        <is>
+          <t>Retention by (pno, ct, gt, pkg_bucket)  —  Override column takes priority. Fallback: pkg_bucket=ALL (dim-level), then global pno default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Fallback hierarchy: Level1=(pno,ct,gt,pkg) pool&gt;=15  →  Level2=(pno,ct,gt) ALL  →  Level3=global(pno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>pno</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>ct</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>gt</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>pkg_bucket</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>n_pool</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Note / Source</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="35" t="n">
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="18" t="n">
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>0.1781</v>
+      </c>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>data pool=73 sec=13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>0.2698</v>
+      </c>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="17" t="n">
+        <v>367</v>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>data pool=367 sec=99</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>0.3208</v>
+      </c>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="17" t="n">
+        <v>53</v>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>data pool=53 sec=17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" s="36" t="n">
+        <v>0.4691</v>
+      </c>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="17" t="n">
+        <v>81</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>data pool=81 sec=38</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>0.2818</v>
+      </c>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="17" t="n">
+        <v>181</v>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>data pool=181 sec=51</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" s="36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>data pool=50 sec=30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>0.2923</v>
+      </c>
+      <c r="F10" s="18" t="n"/>
+      <c r="G10" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>data pool=65 sec=19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>0.2083</v>
+      </c>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="17" t="n">
+        <v>144</v>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>data pool=144 sec=30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>0.2661</v>
+      </c>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="17" t="n">
+        <v>872</v>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>data pool=872 sec=232</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" s="36" t="n">
+        <v>0.3426</v>
+      </c>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="17" t="n">
+        <v>108</v>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>data pool=108 sec=37</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E14" s="36" t="n">
+        <v>0.4795</v>
+      </c>
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="17" t="n">
+        <v>171</v>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>data pool=171 sec=82</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="E15" s="36" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="17" t="n">
+        <v>216</v>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>data pool=216 sec=62</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>0.2358</v>
+      </c>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="17" t="n">
+        <v>335</v>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>data pool=335 sec=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="36" t="n">
+        <v>0.2624</v>
+      </c>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="17" t="n">
+        <v>1719</v>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>data pool=1719 sec=451</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>0.2472</v>
+      </c>
+      <c r="F18" s="18" t="n"/>
+      <c r="G18" s="17" t="n">
+        <v>267</v>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>data pool=267 sec=66</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="A19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="36" t="n">
+        <v>0.4241</v>
+      </c>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="17" t="n">
+        <v>323</v>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>data pool=323 sec=137</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" s="36" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="F20" s="18" t="n"/>
+      <c r="G20" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>data pool=30 sec=8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="E21" s="36" t="n">
+        <v>0.2667</v>
+      </c>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="17" t="n">
+        <v>941</v>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>data pool=941 sec=251</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="A22" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <v>0.3893</v>
+      </c>
+      <c r="F22" s="18" t="n"/>
+      <c r="G22" s="17" t="n">
+        <v>149</v>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>data pool=149 sec=58</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1">
+      <c r="A23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="n">
+        <v>56</v>
+      </c>
+      <c r="E23" s="36" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>data pool=18 sec=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14" customHeight="1">
+      <c r="A24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>0.3022</v>
+      </c>
+      <c r="F24" s="18" t="n"/>
+      <c r="G24" s="17" t="n">
+        <v>268</v>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>data pool=268 sec=81</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14" customHeight="1">
+      <c r="A25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="E25" s="36" t="n">
+        <v>0.1579</v>
+      </c>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>data pool=19 sec=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="A26" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <v>0.4118</v>
+      </c>
+      <c r="F26" s="18" t="n"/>
+      <c r="G26" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>data pool=51 sec=21</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="14" customHeight="1">
+      <c r="A27" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" s="36" t="n">
+        <v>0.5263</v>
+      </c>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="21" t="n">
+        <v>57</v>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>data pool=57 sec=30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="14" customHeight="1">
+      <c r="A28" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E28" s="36" t="n">
+        <v>0.8293</v>
+      </c>
+      <c r="F28" s="18" t="n"/>
+      <c r="G28" s="21" t="n">
+        <v>41</v>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>data pool=41 sec=34</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="14" customHeight="1">
+      <c r="A29" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E29" s="36" t="n">
+        <v>0.4255</v>
+      </c>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="21" t="n">
+        <v>47</v>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>data pool=47 sec=20</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="14" customHeight="1">
+      <c r="A30" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E30" s="36" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>data pool=16 sec=11</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="14" customHeight="1">
+      <c r="A31" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" s="36" t="n">
+        <v>0.3793</v>
+      </c>
+      <c r="F31" s="18" t="n"/>
+      <c r="G31" s="21" t="n">
+        <v>58</v>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>data pool=58 sec=22</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="14" customHeight="1">
+      <c r="A32" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="21" t="n">
+        <v>105</v>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>data pool=105 sec=63</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="14" customHeight="1">
+      <c r="A33" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" s="36" t="n">
+        <v>0.7121</v>
+      </c>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="21" t="n">
+        <v>66</v>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>data pool=66 sec=47</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="14" customHeight="1">
+      <c r="A34" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="36" t="n">
+        <v>0.6264</v>
+      </c>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="21" t="n">
+        <v>91</v>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>data pool=91 sec=57</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="14" customHeight="1">
+      <c r="A35" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E35" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="21" t="n">
+        <v>35</v>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>data pool=35 sec=14</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="14" customHeight="1">
+      <c r="A36" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C36" s="20" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <v>0.2647</v>
+      </c>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="21" t="n">
+        <v>34</v>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>data pool=34 sec=9</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="14" customHeight="1">
+      <c r="A37" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E37" s="36" t="n">
+        <v>0.6052999999999999</v>
+      </c>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="21" t="n">
+        <v>337</v>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>data pool=337 sec=204</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="14" customHeight="1">
+      <c r="A38" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" s="36" t="n">
+        <v>0.7421</v>
+      </c>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="21" t="n">
+        <v>221</v>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>data pool=221 sec=164</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="14" customHeight="1">
+      <c r="A39" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E39" s="36" t="n">
+        <v>0.4538</v>
+      </c>
+      <c r="F39" s="18" t="n"/>
+      <c r="G39" s="21" t="n">
+        <v>260</v>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>data pool=260 sec=118</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="14" customHeight="1">
+      <c r="A40" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C40" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E40" s="36" t="n">
+        <v>0.5443</v>
+      </c>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="21" t="n">
+        <v>79</v>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>data pool=79 sec=43</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="14" customHeight="1">
+      <c r="A41" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="n">
+        <v>24</v>
+      </c>
+      <c r="E41" s="36" t="n">
+        <v>0.3383</v>
+      </c>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="21" t="n">
+        <v>337</v>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>data pool=337 sec=114</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
+      <c r="A42" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C42" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D42" s="21" t="n">
+        <v>32</v>
+      </c>
+      <c r="E42" s="36" t="n">
+        <v>0.5652</v>
+      </c>
+      <c r="F42" s="18" t="n"/>
+      <c r="G42" s="21" t="n">
+        <v>368</v>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>data pool=368 sec=208</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="14" customHeight="1">
+      <c r="A43" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="E43" s="36" t="n">
+        <v>0.4694</v>
+      </c>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="21" t="n">
+        <v>49</v>
+      </c>
+      <c r="H43" s="19" t="inlineStr">
+        <is>
+          <t>data pool=49 sec=23</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="14" customHeight="1">
+      <c r="A44" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C44" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="n">
+        <v>56</v>
+      </c>
+      <c r="E44" s="36" t="n">
+        <v>0.2899</v>
+      </c>
+      <c r="F44" s="18" t="n"/>
+      <c r="G44" s="21" t="n">
+        <v>69</v>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
+        <is>
+          <t>data pool=69 sec=20</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="14" customHeight="1">
+      <c r="A45" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D45" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" s="36" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F45" s="18" t="n"/>
+      <c r="G45" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>data pool=32 sec=24</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="14" customHeight="1">
+      <c r="A46" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="E46" s="36" t="n">
+        <v>0.5667</v>
+      </c>
+      <c r="F46" s="18" t="n"/>
+      <c r="G46" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="H46" s="19" t="inlineStr">
+        <is>
+          <t>data pool=30 sec=17</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="14" customHeight="1">
+      <c r="A47" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D47" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="E47" s="36" t="n">
+        <v>0.6341</v>
+      </c>
+      <c r="F47" s="18" t="n"/>
+      <c r="G47" s="23" t="n">
+        <v>41</v>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>data pool=41 sec=26</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="14" customHeight="1">
+      <c r="A48" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D48" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E48" s="36" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="F48" s="18" t="n"/>
+      <c r="G48" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="H48" s="19" t="inlineStr">
+        <is>
+          <t>data pool=32 sec=28</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="14" customHeight="1">
+      <c r="A49" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D49" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E49" s="36" t="n">
+        <v>0.7696</v>
+      </c>
+      <c r="F49" s="18" t="n"/>
+      <c r="G49" s="23" t="n">
+        <v>230</v>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>data pool=230 sec=177</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" s="36" t="n">
+        <v>0.6812</v>
+      </c>
+      <c r="F50" s="18" t="n"/>
+      <c r="G50" s="23" t="n">
+        <v>69</v>
+      </c>
+      <c r="H50" s="19" t="inlineStr">
+        <is>
+          <t>data pool=69 sec=47</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="14" customHeight="1">
+      <c r="A51" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="E51" s="36" t="n">
+        <v>0.6329</v>
+      </c>
+      <c r="F51" s="18" t="n"/>
+      <c r="G51" s="23" t="n">
+        <v>158</v>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>data pool=158 sec=100</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="14" customHeight="1">
+      <c r="A52" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D52" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E52" s="36" t="n">
+        <v>0.6765</v>
+      </c>
+      <c r="F52" s="18" t="n"/>
+      <c r="G52" s="23" t="n">
+        <v>34</v>
+      </c>
+      <c r="H52" s="19" t="inlineStr">
+        <is>
+          <t>data pool=34 sec=23</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="14" customHeight="1">
+      <c r="A53" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D53" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="E53" s="36" t="n">
+        <v>0.6042</v>
+      </c>
+      <c r="F53" s="18" t="n"/>
+      <c r="G53" s="23" t="n">
+        <v>48</v>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>data pool=48 sec=29</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="14" customHeight="1">
+      <c r="A54" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B54" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="E54" s="36" t="n">
+        <v>0.6818</v>
+      </c>
+      <c r="F54" s="18" t="n"/>
+      <c r="G54" s="23" t="n">
+        <v>198</v>
+      </c>
+      <c r="H54" s="19" t="inlineStr">
+        <is>
+          <t>data pool=198 sec=135</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="14" customHeight="1">
+      <c r="A55" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E55" s="36" t="n">
+        <v>0.6818</v>
+      </c>
+      <c r="F55" s="18" t="n"/>
+      <c r="G55" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>data pool=22 sec=15</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="14" customHeight="1">
+      <c r="A56" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C56" s="24" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="E56" s="36" t="n">
+        <v>0.7727000000000001</v>
+      </c>
+      <c r="F56" s="18" t="n"/>
+      <c r="G56" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="H56" s="19" t="inlineStr">
+        <is>
+          <t>data pool=22 sec=17</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="14" customHeight="1">
+      <c r="A57" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C57" s="24" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E57" s="36" t="n">
+        <v>0.5862000000000001</v>
+      </c>
+      <c r="F57" s="18" t="n"/>
+      <c r="G57" s="25" t="n">
+        <v>29</v>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>data pool=29 sec=17</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="14" customHeight="1">
+      <c r="A58" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C58" s="24" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D58" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E58" s="36" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="F58" s="18" t="n"/>
+      <c r="G58" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
+        <is>
+          <t>data pool=16 sec=13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="14" customHeight="1">
+      <c r="A59" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C59" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D59" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E59" s="36" t="n">
+        <v>0.6939</v>
+      </c>
+      <c r="F59" s="18" t="n"/>
+      <c r="G59" s="25" t="n">
+        <v>147</v>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>data pool=147 sec=102</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="14" customHeight="1">
+      <c r="A60" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C60" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D60" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E60" s="36" t="n">
+        <v>0.4894</v>
+      </c>
+      <c r="F60" s="18" t="n"/>
+      <c r="G60" s="25" t="n">
+        <v>47</v>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>data pool=47 sec=23</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="14" customHeight="1">
+      <c r="A61" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C61" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D61" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="E61" s="36" t="n">
+        <v>0.6465</v>
+      </c>
+      <c r="F61" s="18" t="n"/>
+      <c r="G61" s="25" t="n">
+        <v>99</v>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>data pool=99 sec=64</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="14" customHeight="1">
+      <c r="A62" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C62" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D62" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E62" s="36" t="n">
+        <v>0.8077</v>
+      </c>
+      <c r="F62" s="18" t="n"/>
+      <c r="G62" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>data pool=26 sec=21</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="14" customHeight="1">
+      <c r="A63" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B63" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C63" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E63" s="36" t="n">
+        <v>0.6129</v>
+      </c>
+      <c r="F63" s="18" t="n"/>
+      <c r="G63" s="25" t="n">
+        <v>31</v>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>data pool=31 sec=19</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="14" customHeight="1">
+      <c r="A64" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B64" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C64" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E64" s="36" t="n">
+        <v>0.9137999999999999</v>
+      </c>
+      <c r="F64" s="18" t="n"/>
+      <c r="G64" s="25" t="n">
+        <v>58</v>
+      </c>
+      <c r="H64" s="19" t="inlineStr">
+        <is>
+          <t>data pool=58 sec=53</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="14" customHeight="1">
+      <c r="A65" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D65" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E65" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="18" t="n"/>
+      <c r="G65" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="H65" s="19" t="inlineStr">
+        <is>
+          <t>data pool=18 sec=18</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="14" customHeight="1">
+      <c r="A66" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B66" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D66" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" s="36" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="F66" s="18" t="n"/>
+      <c r="G66" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="H66" s="19" t="inlineStr">
+        <is>
+          <t>data pool=16 sec=13</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="14" customHeight="1">
+      <c r="A67" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C67" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D67" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E67" s="36" t="n">
+        <v>0.8941</v>
+      </c>
+      <c r="F67" s="18" t="n"/>
+      <c r="G67" s="27" t="n">
+        <v>85</v>
+      </c>
+      <c r="H67" s="19" t="inlineStr">
+        <is>
+          <t>data pool=85 sec=76</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="14" customHeight="1">
+      <c r="A68" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B68" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C68" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D68" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" s="36" t="n">
+        <v>0.8235</v>
+      </c>
+      <c r="F68" s="18" t="n"/>
+      <c r="G68" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="H68" s="19" t="inlineStr">
+        <is>
+          <t>data pool=17 sec=14</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="14" customHeight="1">
+      <c r="A69" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B69" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C69" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="n">
+        <v>16</v>
+      </c>
+      <c r="E69" s="36" t="n">
+        <v>0.8929</v>
+      </c>
+      <c r="F69" s="18" t="n"/>
+      <c r="G69" s="27" t="n">
+        <v>56</v>
+      </c>
+      <c r="H69" s="19" t="inlineStr">
+        <is>
+          <t>data pool=56 sec=50</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="14" customHeight="1">
+      <c r="A70" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B70" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D70" s="27" t="n">
+        <v>24</v>
+      </c>
+      <c r="E70" s="36" t="n">
+        <v>0.2941</v>
+      </c>
+      <c r="F70" s="18" t="n"/>
+      <c r="G70" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="H70" s="19" t="inlineStr">
+        <is>
+          <t>data pool=17 sec=5</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="14" customHeight="1">
+      <c r="A71" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B71" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C71" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D71" s="27" t="n">
+        <v>32</v>
+      </c>
+      <c r="E71" s="36" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="F71" s="18" t="n"/>
+      <c r="G71" s="27" t="n">
+        <v>18</v>
+      </c>
+      <c r="H71" s="19" t="inlineStr">
+        <is>
+          <t>data pool=18 sec=14</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="14" customHeight="1">
+      <c r="A72" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B72" s="28" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C72" s="28" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="D72" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E72" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F72" s="18" t="n"/>
+      <c r="G72" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="H72" s="19" t="inlineStr">
+        <is>
+          <t>data pool=20 sec=16</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="14" customHeight="1">
+      <c r="A73" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" s="28" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C73" s="28" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D73" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="E73" s="36" t="n">
+        <v>0.9296</v>
+      </c>
+      <c r="F73" s="18" t="n"/>
+      <c r="G73" s="29" t="n">
+        <v>71</v>
+      </c>
+      <c r="H73" s="19" t="inlineStr">
+        <is>
+          <t>data pool=71 sec=66</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="14" customHeight="1">
+      <c r="A74" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B74" s="28" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C74" s="28" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D74" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="E74" s="36" t="n">
+        <v>0.7917</v>
+      </c>
+      <c r="F74" s="18" t="n"/>
+      <c r="G74" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="H74" s="19" t="inlineStr">
+        <is>
+          <t>data pool=24 sec=19</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="14" customHeight="1">
+      <c r="A75" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D75" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E75" s="36" t="n">
+        <v>0.8696</v>
+      </c>
+      <c r="F75" s="18" t="n"/>
+      <c r="G75" s="17" t="n">
+        <v>46</v>
+      </c>
+      <c r="H75" s="19" t="inlineStr">
+        <is>
+          <t>data pool=46 sec=40</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="14" customHeight="1">
+      <c r="A76" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B76" s="20" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D76" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E76" s="36" t="n">
+        <v>0.7838000000000001</v>
+      </c>
+      <c r="F76" s="18" t="n"/>
+      <c r="G76" s="21" t="n">
+        <v>37</v>
+      </c>
+      <c r="H76" s="19" t="inlineStr">
+        <is>
+          <t>data pool=37 sec=29</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="14" customHeight="1">
+      <c r="A77" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B77" s="22" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D77" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E77" s="36" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="F77" s="18" t="n"/>
+      <c r="G77" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="H77" s="19" t="inlineStr">
+        <is>
+          <t>data pool=32 sec=31</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="14" customHeight="1">
+      <c r="A78" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D78" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E78" s="36" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F78" s="18" t="n"/>
+      <c r="G78" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="H78" s="19" t="inlineStr">
+        <is>
+          <t>data pool=25 sec=22</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="14" customHeight="1">
+      <c r="A79" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B79" s="26" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="C79" s="26" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D79" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E79" s="36" t="n">
+        <v>0.8696</v>
+      </c>
+      <c r="F79" s="18" t="n"/>
+      <c r="G79" s="27" t="n">
+        <v>23</v>
+      </c>
+      <c r="H79" s="19" t="inlineStr">
+        <is>
+          <t>data pool=23 sec=20</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="A80" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B80" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C80" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D80" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E80" s="18" t="n">
         <v>0.2903</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="F80" s="18" t="n"/>
+      <c r="G80" s="39" t="n">
         <v>6648</v>
       </c>
-      <c r="D3" s="17" t="n">
-        <v>1930</v>
-      </c>
-      <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>data pool=6648 sec=1930</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="36" t="n">
+      <c r="H80" s="19" t="inlineStr">
+        <is>
+          <t>data pool=6648 sec=1930  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B81" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C81" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D81" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="n">
         <v>0.5292</v>
       </c>
-      <c r="C4" s="21" t="n">
+      <c r="F81" s="18" t="n"/>
+      <c r="G81" s="39" t="n">
         <v>2432</v>
       </c>
-      <c r="D4" s="21" t="n">
-        <v>1287</v>
-      </c>
-      <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>data pool=2432 sec=1287</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="37" t="n">
+      <c r="H81" s="19" t="inlineStr">
+        <is>
+          <t>data pool=2432 sec=1287  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B82" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C82" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D82" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E82" s="18" t="n">
         <v>0.6934</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="F82" s="18" t="n"/>
+      <c r="G82" s="39" t="n">
         <v>972</v>
       </c>
-      <c r="D5" s="23" t="n">
-        <v>674</v>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>data pool=972 sec=674</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="38" t="n">
+      <c r="H82" s="19" t="inlineStr">
+        <is>
+          <t>data pool=972 sec=674  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B83" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C83" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D83" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E83" s="18" t="n">
         <v>0.6953</v>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="F83" s="18" t="n"/>
+      <c r="G83" s="39" t="n">
         <v>535</v>
       </c>
-      <c r="D6" s="25" t="n">
-        <v>372</v>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>data pool=535 sec=372</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="39" t="n">
+      <c r="H83" s="19" t="inlineStr">
+        <is>
+          <t>data pool=535 sec=372  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B84" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C84" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D84" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E84" s="18" t="n">
         <v>0.8566</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="F84" s="18" t="n"/>
+      <c r="G84" s="39" t="n">
         <v>258</v>
       </c>
-      <c r="D7" s="27" t="n">
-        <v>221</v>
-      </c>
-      <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>data pool=258 sec=221</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="40" t="n">
+      <c r="H84" s="19" t="inlineStr">
+        <is>
+          <t>data pool=258 sec=221  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B85" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C85" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D85" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E85" s="18" t="n">
         <v>0.8652</v>
       </c>
-      <c r="C8" s="29" t="n">
+      <c r="F85" s="18" t="n"/>
+      <c r="G85" s="39" t="n">
         <v>178</v>
       </c>
-      <c r="D8" s="29" t="n">
-        <v>154</v>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>data pool=178 sec=154</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="35" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="18" t="n">
+      <c r="H85" s="19" t="inlineStr">
+        <is>
+          <t>data pool=178 sec=154  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B86" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C86" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D86" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E86" s="18" t="n">
         <v>0.8532</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="F86" s="18" t="n"/>
+      <c r="G86" s="39" t="n">
         <v>109</v>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>93</v>
-      </c>
-      <c r="E9" s="19" t="inlineStr">
-        <is>
-          <t>data pool=109 sec=93</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="36" t="n">
+      <c r="H86" s="19" t="inlineStr">
+        <is>
+          <t>data pool=109 sec=93  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="37" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B87" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C87" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D87" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E87" s="18" t="n">
         <v>0.8594000000000001</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="F87" s="18" t="n"/>
+      <c r="G87" s="39" t="n">
         <v>64</v>
       </c>
-      <c r="D10" s="21" t="n">
-        <v>55</v>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>data pool=64 sec=55</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="37" t="n">
+      <c r="H87" s="19" t="inlineStr">
+        <is>
+          <t>data pool=64 sec=55  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" s="37" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B88" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C88" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D88" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E88" s="18" t="n">
         <v>0.8511</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="F88" s="18" t="n"/>
+      <c r="G88" s="39" t="n">
         <v>47</v>
       </c>
-      <c r="D11" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>data pool=47 sec=40</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="38" t="n">
+      <c r="H88" s="19" t="inlineStr">
+        <is>
+          <t>data pool=47 sec=40  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="37" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B89" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C89" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D89" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="n">
         <v>0.8611</v>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="F89" s="18" t="n"/>
+      <c r="G89" s="39" t="n">
         <v>36</v>
       </c>
-      <c r="D12" s="25" t="n">
-        <v>31</v>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>data pool=36 sec=31</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="39" t="n">
+      <c r="H89" s="19" t="inlineStr">
+        <is>
+          <t>data pool=36 sec=31  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="37" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B90" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C90" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D90" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E90" s="18" t="n">
         <v>0.8788</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="F90" s="18" t="n"/>
+      <c r="G90" s="39" t="n">
         <v>33</v>
       </c>
-      <c r="D13" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>data pool=33 sec=29</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="40" t="n">
+      <c r="H90" s="19" t="inlineStr">
+        <is>
+          <t>data pool=33 sec=29  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="37" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B91" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C91" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E91" s="18" t="n">
         <v>0.8</v>
       </c>
-      <c r="C14" s="29" t="n">
+      <c r="F91" s="18" t="n"/>
+      <c r="G91" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="D14" s="29" t="n">
-        <v>16</v>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>data pool=20 sec=16</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="35" t="n">
+      <c r="H91" s="19" t="inlineStr">
+        <is>
+          <t>data pool=20 sec=16  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15" customHeight="1">
+      <c r="A92" s="37" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B92" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C92" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D92" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E92" s="18" t="n">
         <v>0.8182</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="F92" s="18" t="n"/>
+      <c r="G92" s="39" t="n">
         <v>11</v>
       </c>
-      <c r="D15" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>data pool=11 sec=9</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="36" t="n">
+      <c r="H92" s="19" t="inlineStr">
+        <is>
+          <t>data pool=11 sec=9  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="37" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B93" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C93" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D93" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E93" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="F93" s="18" t="n"/>
+      <c r="G93" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="D16" s="21" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>data pool=10 sec=9</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="37" t="n">
+      <c r="H93" s="19" t="inlineStr">
+        <is>
+          <t>data pool=10 sec=9  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B94" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="C94" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="D94" s="38" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="n">
         <v>0.72</v>
       </c>
-      <c r="C17" s="41" t="inlineStr">
+      <c r="F94" s="18" t="n"/>
+      <c r="G94" s="40" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D17" s="41" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>hardcoded default (pool=6&lt;10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="34" t="inlineStr">
-        <is>
-          <t>payment_no 1 = primary (not secondary). pno 2 = first renewal. For pno &gt;= 16 the model uses RETENTION_PNO_HIGH = 72.0%.</t>
-        </is>
-      </c>
-      <c r="B19" s="59" t="n"/>
-      <c r="C19" s="59" t="n"/>
-      <c r="D19" s="59" t="n"/>
-      <c r="E19" s="60" t="n"/>
+      <c r="H94" s="19" t="inlineStr">
+        <is>
+          <t>hardcoded default (pool=6&lt;10)  ← Level-2 fallback (ALL pkg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="36" customHeight="1">
+      <c r="A96" s="34" t="inlineStr">
+        <is>
+          <t>pno=1 = primary (not secondary). pno=2 = first renewal. Override (col F) takes priority over Retention (col E) if non-empty. pkg_bucket rows = Level-1 (pool&gt;=15). ALL rows = Level-2 fallback. For pno&gt;=16 model uses RETENTION_PNO_HIGH=72.0%.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A19:E19"/>
+  <mergeCells count="3">
+    <mergeCell ref="A96:H96"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15965,8 +18362,6 @@
           <t>Segment Shares  —  EDIT yellow column (must sum to 1.0 across all 4 segments)</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15986,7 +18381,7 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="42" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
@@ -16001,7 +18396,7 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Earlier</t>
         </is>
@@ -16016,7 +18411,7 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>Reanim</t>
         </is>
@@ -16031,7 +18426,7 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="45" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>Upgrades</t>
         </is>
@@ -16051,7 +18446,7 @@
           <t>SUM</t>
         </is>
       </c>
-      <c r="B7" s="46" t="n">
+      <c r="B7" s="45" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="28" t="inlineStr">
@@ -16066,8 +18461,6 @@
           <t>Edit yellow cells. The model normalizes shares automatically if sum != 1.0.</t>
         </is>
       </c>
-      <c r="B9" s="59" t="n"/>
-      <c r="C9" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -16101,11 +18494,6 @@
           <t>Ext-curve (Lag Curve for Future Cohorts)  —  EDIT col E (Override) only if needed</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="59" t="n"/>
-      <c r="E1" s="59" t="n"/>
-      <c r="F1" s="60" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -16113,11 +18501,6 @@
           <t>Recent (2024-01 to 2025-06): lags 1-22  |  Full fallback (2023-01 to 2025-06): lags 23-33  |  Used by mode=ext (Jun-Dec 2026)</t>
         </is>
       </c>
-      <c r="B2" s="59" t="n"/>
-      <c r="C2" s="59" t="n"/>
-      <c r="D2" s="59" t="n"/>
-      <c r="E2" s="59" t="n"/>
-      <c r="F2" s="60" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -16152,748 +18535,748 @@
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="47" t="inlineStr">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>lag 1</t>
         </is>
       </c>
-      <c r="B4" s="48" t="n">
+      <c r="B4" s="47" t="n">
         <v>0.03243981260767305</v>
       </c>
-      <c r="C4" s="48" t="n">
+      <c r="C4" s="47" t="n">
         <v>0.03325380378132611</v>
       </c>
-      <c r="D4" s="49" t="n">
+      <c r="D4" s="48" t="n">
         <v>0.03325380378132611</v>
       </c>
-      <c r="E4" s="50" t="inlineStr"/>
-      <c r="F4" s="51" t="inlineStr">
+      <c r="E4" s="49" t="inlineStr"/>
+      <c r="F4" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="47" t="inlineStr">
+      <c r="A5" s="46" t="inlineStr">
         <is>
           <t>lag 2</t>
         </is>
       </c>
-      <c r="B5" s="48" t="n">
+      <c r="B5" s="47" t="n">
         <v>0.05565081335823394</v>
       </c>
-      <c r="C5" s="48" t="n">
+      <c r="C5" s="47" t="n">
         <v>0.05229594677145271</v>
       </c>
-      <c r="D5" s="49" t="n">
+      <c r="D5" s="48" t="n">
         <v>0.05229594677145271</v>
       </c>
-      <c r="E5" s="50" t="inlineStr"/>
-      <c r="F5" s="51" t="inlineStr">
+      <c r="E5" s="49" t="inlineStr"/>
+      <c r="F5" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="47" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>lag 3</t>
         </is>
       </c>
-      <c r="B6" s="48" t="n">
+      <c r="B6" s="47" t="n">
         <v>0.05740292312901271</v>
       </c>
-      <c r="C6" s="48" t="n">
+      <c r="C6" s="47" t="n">
         <v>0.04043051008979147</v>
       </c>
-      <c r="D6" s="49" t="n">
+      <c r="D6" s="48" t="n">
         <v>0.04043051008979147</v>
       </c>
-      <c r="E6" s="50" t="inlineStr"/>
-      <c r="F6" s="51" t="inlineStr">
+      <c r="E6" s="49" t="inlineStr"/>
+      <c r="F6" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="47" t="inlineStr">
+      <c r="A7" s="46" t="inlineStr">
         <is>
           <t>lag 4</t>
         </is>
       </c>
-      <c r="B7" s="48" t="n">
+      <c r="B7" s="47" t="n">
         <v>0.08721467251692649</v>
       </c>
-      <c r="C7" s="48" t="n">
+      <c r="C7" s="47" t="n">
         <v>0.06933519380542201</v>
       </c>
-      <c r="D7" s="49" t="n">
+      <c r="D7" s="48" t="n">
         <v>0.06933519380542201</v>
       </c>
-      <c r="E7" s="50" t="inlineStr"/>
-      <c r="F7" s="51" t="inlineStr">
+      <c r="E7" s="49" t="inlineStr"/>
+      <c r="F7" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
-      <c r="A8" s="47" t="inlineStr">
+      <c r="A8" s="46" t="inlineStr">
         <is>
           <t>lag 5</t>
         </is>
       </c>
-      <c r="B8" s="48" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.04908093490622328</v>
       </c>
-      <c r="C8" s="48" t="n">
+      <c r="C8" s="47" t="n">
         <v>0.04150558638908253</v>
       </c>
-      <c r="D8" s="49" t="n">
+      <c r="D8" s="48" t="n">
         <v>0.04150558638908253</v>
       </c>
-      <c r="E8" s="50" t="inlineStr"/>
-      <c r="F8" s="51" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr"/>
+      <c r="F8" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
-      <c r="A9" s="47" t="inlineStr">
+      <c r="A9" s="46" t="inlineStr">
         <is>
           <t>lag 6</t>
         </is>
       </c>
-      <c r="B9" s="48" t="n">
+      <c r="B9" s="47" t="n">
         <v>0.04107542987799979</v>
       </c>
-      <c r="C9" s="48" t="n">
+      <c r="C9" s="47" t="n">
         <v>0.03334841325604449</v>
       </c>
-      <c r="D9" s="49" t="n">
+      <c r="D9" s="48" t="n">
         <v>0.03334841325604449</v>
       </c>
-      <c r="E9" s="50" t="inlineStr"/>
-      <c r="F9" s="51" t="inlineStr">
+      <c r="E9" s="49" t="inlineStr"/>
+      <c r="F9" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="47" t="inlineStr">
+      <c r="A10" s="46" t="inlineStr">
         <is>
           <t>lag 7</t>
         </is>
       </c>
-      <c r="B10" s="48" t="n">
+      <c r="B10" s="47" t="n">
         <v>0.04132556188857849</v>
       </c>
-      <c r="C10" s="48" t="n">
+      <c r="C10" s="47" t="n">
         <v>0.04115337003794277</v>
       </c>
-      <c r="D10" s="49" t="n">
+      <c r="D10" s="48" t="n">
         <v>0.04115337003794277</v>
       </c>
-      <c r="E10" s="50" t="inlineStr"/>
-      <c r="F10" s="51" t="inlineStr">
+      <c r="E10" s="49" t="inlineStr"/>
+      <c r="F10" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="47" t="inlineStr">
+      <c r="A11" s="46" t="inlineStr">
         <is>
           <t>lag 8</t>
         </is>
       </c>
-      <c r="B11" s="48" t="n">
+      <c r="B11" s="47" t="n">
         <v>0.07794682286006098</v>
       </c>
-      <c r="C11" s="48" t="n">
+      <c r="C11" s="47" t="n">
         <v>0.08012093056296371</v>
       </c>
-      <c r="D11" s="49" t="n">
+      <c r="D11" s="48" t="n">
         <v>0.08012093056296371</v>
       </c>
-      <c r="E11" s="50" t="inlineStr"/>
-      <c r="F11" s="51" t="inlineStr">
+      <c r="E11" s="49" t="inlineStr"/>
+      <c r="F11" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="47" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>lag 9</t>
         </is>
       </c>
-      <c r="B12" s="48" t="n">
+      <c r="B12" s="47" t="n">
         <v>0.05219903571086893</v>
       </c>
-      <c r="C12" s="48" t="n">
+      <c r="C12" s="47" t="n">
         <v>0.0463728113540315</v>
       </c>
-      <c r="D12" s="49" t="n">
+      <c r="D12" s="48" t="n">
         <v>0.0463728113540315</v>
       </c>
-      <c r="E12" s="50" t="inlineStr"/>
-      <c r="F12" s="51" t="inlineStr">
+      <c r="E12" s="49" t="inlineStr"/>
+      <c r="F12" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="47" t="inlineStr">
+      <c r="A13" s="46" t="inlineStr">
         <is>
           <t>lag 10</t>
         </is>
       </c>
-      <c r="B13" s="48" t="n">
+      <c r="B13" s="47" t="n">
         <v>0.0263084995491605</v>
       </c>
-      <c r="C13" s="48" t="n">
+      <c r="C13" s="47" t="n">
         <v>0.02540345997477899</v>
       </c>
-      <c r="D13" s="49" t="n">
+      <c r="D13" s="48" t="n">
         <v>0.02540345997477899</v>
       </c>
-      <c r="E13" s="50" t="inlineStr"/>
-      <c r="F13" s="51" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr"/>
+      <c r="F13" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="47" t="inlineStr">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>lag 11</t>
         </is>
       </c>
-      <c r="B14" s="48" t="n">
+      <c r="B14" s="47" t="n">
         <v>0.01694534590044715</v>
       </c>
-      <c r="C14" s="48" t="n">
+      <c r="C14" s="47" t="n">
         <v>0.01670792262887267</v>
       </c>
-      <c r="D14" s="49" t="n">
+      <c r="D14" s="48" t="n">
         <v>0.01670792262887267</v>
       </c>
-      <c r="E14" s="50" t="inlineStr"/>
-      <c r="F14" s="51" t="inlineStr">
+      <c r="E14" s="49" t="inlineStr"/>
+      <c r="F14" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="47" t="inlineStr">
+      <c r="A15" s="46" t="inlineStr">
         <is>
           <t>lag 12</t>
         </is>
       </c>
-      <c r="B15" s="48" t="n">
+      <c r="B15" s="47" t="n">
         <v>0.02311776204827275</v>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="47" t="n">
         <v>0.0203014383813916</v>
       </c>
-      <c r="D15" s="49" t="n">
+      <c r="D15" s="48" t="n">
         <v>0.0203014383813916</v>
       </c>
-      <c r="E15" s="50" t="inlineStr"/>
-      <c r="F15" s="51" t="inlineStr">
+      <c r="E15" s="49" t="inlineStr"/>
+      <c r="F15" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="47" t="inlineStr">
+      <c r="A16" s="46" t="inlineStr">
         <is>
           <t>lag 13</t>
         </is>
       </c>
-      <c r="B16" s="48" t="n">
+      <c r="B16" s="47" t="n">
         <v>0.02009059602064579</v>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="47" t="n">
         <v>0.0129558204440133</v>
       </c>
-      <c r="D16" s="49" t="n">
+      <c r="D16" s="48" t="n">
         <v>0.0129558204440133</v>
       </c>
-      <c r="E16" s="50" t="inlineStr"/>
-      <c r="F16" s="51" t="inlineStr">
+      <c r="E16" s="49" t="inlineStr"/>
+      <c r="F16" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="47" t="inlineStr">
+      <c r="A17" s="46" t="inlineStr">
         <is>
           <t>lag 14</t>
         </is>
       </c>
-      <c r="B17" s="48" t="n">
+      <c r="B17" s="47" t="n">
         <v>0.01442047607706917</v>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="47" t="n">
         <v>0.0123686957085169</v>
       </c>
-      <c r="D17" s="49" t="n">
+      <c r="D17" s="48" t="n">
         <v>0.0123686957085169</v>
       </c>
-      <c r="E17" s="50" t="inlineStr"/>
-      <c r="F17" s="51" t="inlineStr">
+      <c r="E17" s="49" t="inlineStr"/>
+      <c r="F17" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="47" t="inlineStr">
+      <c r="A18" s="46" t="inlineStr">
         <is>
           <t>lag 15</t>
         </is>
       </c>
-      <c r="B18" s="48" t="n">
+      <c r="B18" s="47" t="n">
         <v>0.0190650878142931</v>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="47" t="n">
         <v>0.02177364537386275</v>
       </c>
-      <c r="D18" s="49" t="n">
+      <c r="D18" s="48" t="n">
         <v>0.02177364537386275</v>
       </c>
-      <c r="E18" s="50" t="inlineStr"/>
-      <c r="F18" s="51" t="inlineStr">
+      <c r="E18" s="49" t="inlineStr"/>
+      <c r="F18" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="47" t="inlineStr">
+      <c r="A19" s="46" t="inlineStr">
         <is>
           <t>lag 16</t>
         </is>
       </c>
-      <c r="B19" s="48" t="n">
+      <c r="B19" s="47" t="n">
         <v>0.03493600983148009</v>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="47" t="n">
         <v>0.03563806584503205</v>
       </c>
-      <c r="D19" s="49" t="n">
+      <c r="D19" s="48" t="n">
         <v>0.03563806584503205</v>
       </c>
-      <c r="E19" s="50" t="inlineStr"/>
-      <c r="F19" s="51" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr"/>
+      <c r="F19" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="47" t="inlineStr">
+      <c r="A20" s="46" t="inlineStr">
         <is>
           <t>lag 17</t>
         </is>
       </c>
-      <c r="B20" s="48" t="n">
+      <c r="B20" s="47" t="n">
         <v>0.0265347588824575</v>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="47" t="n">
         <v>0.02582494976486335</v>
       </c>
-      <c r="D20" s="49" t="n">
+      <c r="D20" s="48" t="n">
         <v>0.02582494976486335</v>
       </c>
-      <c r="E20" s="50" t="inlineStr"/>
-      <c r="F20" s="51" t="inlineStr">
+      <c r="E20" s="49" t="inlineStr"/>
+      <c r="F20" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="47" t="inlineStr">
+      <c r="A21" s="46" t="inlineStr">
         <is>
           <t>lag 18</t>
         </is>
       </c>
-      <c r="B21" s="48" t="n">
+      <c r="B21" s="47" t="n">
         <v>0.01720805529257647</v>
       </c>
-      <c r="C21" s="48" t="n">
+      <c r="C21" s="47" t="n">
         <v>0.0141590908625448</v>
       </c>
-      <c r="D21" s="49" t="n">
+      <c r="D21" s="48" t="n">
         <v>0.0141590908625448</v>
       </c>
-      <c r="E21" s="50" t="inlineStr"/>
-      <c r="F21" s="51" t="inlineStr">
+      <c r="E21" s="49" t="inlineStr"/>
+      <c r="F21" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="47" t="inlineStr">
+      <c r="A22" s="46" t="inlineStr">
         <is>
           <t>lag 19</t>
         </is>
       </c>
-      <c r="B22" s="48" t="n">
+      <c r="B22" s="47" t="n">
         <v>0.01112484167561391</v>
       </c>
-      <c r="C22" s="48" t="n">
+      <c r="C22" s="47" t="n">
         <v>0.01008889509869752</v>
       </c>
-      <c r="D22" s="49" t="n">
+      <c r="D22" s="48" t="n">
         <v>0.01008889509869752</v>
       </c>
-      <c r="E22" s="50" t="inlineStr"/>
-      <c r="F22" s="51" t="inlineStr">
+      <c r="E22" s="49" t="inlineStr"/>
+      <c r="F22" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="47" t="inlineStr">
+      <c r="A23" s="46" t="inlineStr">
         <is>
           <t>lag 20</t>
         </is>
       </c>
-      <c r="B23" s="48" t="n">
+      <c r="B23" s="47" t="n">
         <v>0.01020671444500314</v>
       </c>
-      <c r="C23" s="48" t="n">
+      <c r="C23" s="47" t="n">
         <v>0.009296585755124544</v>
       </c>
-      <c r="D23" s="49" t="n">
+      <c r="D23" s="48" t="n">
         <v>0.009296585755124544</v>
       </c>
-      <c r="E23" s="50" t="inlineStr"/>
-      <c r="F23" s="51" t="inlineStr">
+      <c r="E23" s="49" t="inlineStr"/>
+      <c r="F23" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="47" t="inlineStr">
+      <c r="A24" s="46" t="inlineStr">
         <is>
           <t>lag 21</t>
         </is>
       </c>
-      <c r="B24" s="48" t="n">
+      <c r="B24" s="47" t="n">
         <v>0.009025071771145076</v>
       </c>
-      <c r="C24" s="48" t="n">
+      <c r="C24" s="47" t="n">
         <v>0.00748335033616986</v>
       </c>
-      <c r="D24" s="49" t="n">
+      <c r="D24" s="48" t="n">
         <v>0.00748335033616986</v>
       </c>
-      <c r="E24" s="50" t="inlineStr"/>
-      <c r="F24" s="51" t="inlineStr">
+      <c r="E24" s="49" t="inlineStr"/>
+      <c r="F24" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="47" t="inlineStr">
+      <c r="A25" s="46" t="inlineStr">
         <is>
           <t>lag 22</t>
         </is>
       </c>
-      <c r="B25" s="48" t="n">
+      <c r="B25" s="47" t="n">
         <v>0.01282232984589626</v>
       </c>
-      <c r="C25" s="48" t="n">
+      <c r="C25" s="47" t="n">
         <v>0.006855762570378132</v>
       </c>
-      <c r="D25" s="49" t="n">
+      <c r="D25" s="48" t="n">
         <v>0.006855762570378132</v>
       </c>
-      <c r="E25" s="50" t="inlineStr"/>
-      <c r="F25" s="51" t="inlineStr">
+      <c r="E25" s="49" t="inlineStr"/>
+      <c r="F25" s="50" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="47" t="inlineStr">
+      <c r="A26" s="46" t="inlineStr">
         <is>
           <t>lag 23</t>
         </is>
       </c>
-      <c r="B26" s="48" t="n">
+      <c r="B26" s="47" t="n">
         <v>0.0111539522300041</v>
       </c>
-      <c r="C26" s="47" t="inlineStr">
+      <c r="C26" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D26" s="52" t="n">
+      <c r="D26" s="51" t="n">
         <v>0.0111539522300041</v>
       </c>
-      <c r="E26" s="50" t="inlineStr"/>
-      <c r="F26" s="51" t="inlineStr">
+      <c r="E26" s="49" t="inlineStr"/>
+      <c r="F26" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="47" t="inlineStr">
+      <c r="A27" s="46" t="inlineStr">
         <is>
           <t>lag 24</t>
         </is>
       </c>
-      <c r="B27" s="48" t="n">
+      <c r="B27" s="47" t="n">
         <v>0.01356349181248091</v>
       </c>
-      <c r="C27" s="47" t="inlineStr">
+      <c r="C27" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D27" s="52" t="n">
+      <c r="D27" s="51" t="n">
         <v>0.01356349181248091</v>
       </c>
-      <c r="E27" s="50" t="inlineStr"/>
-      <c r="F27" s="51" t="inlineStr">
+      <c r="E27" s="49" t="inlineStr"/>
+      <c r="F27" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="47" t="inlineStr">
+      <c r="A28" s="46" t="inlineStr">
         <is>
           <t>lag 25</t>
         </is>
       </c>
-      <c r="B28" s="48" t="n">
+      <c r="B28" s="47" t="n">
         <v>0.01050675670936246</v>
       </c>
-      <c r="C28" s="47" t="inlineStr">
+      <c r="C28" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D28" s="52" t="n">
+      <c r="D28" s="51" t="n">
         <v>0.01050675670936246</v>
       </c>
-      <c r="E28" s="50" t="inlineStr"/>
-      <c r="F28" s="51" t="inlineStr">
+      <c r="E28" s="49" t="inlineStr"/>
+      <c r="F28" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="A29" s="47" t="inlineStr">
+      <c r="A29" s="46" t="inlineStr">
         <is>
           <t>lag 26</t>
         </is>
       </c>
-      <c r="B29" s="48" t="n">
+      <c r="B29" s="47" t="n">
         <v>0.01034430286365552</v>
       </c>
-      <c r="C29" s="47" t="inlineStr">
+      <c r="C29" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D29" s="52" t="n">
+      <c r="D29" s="51" t="n">
         <v>0.01034430286365552</v>
       </c>
-      <c r="E29" s="50" t="inlineStr"/>
-      <c r="F29" s="51" t="inlineStr">
+      <c r="E29" s="49" t="inlineStr"/>
+      <c r="F29" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
-      <c r="A30" s="47" t="inlineStr">
+      <c r="A30" s="46" t="inlineStr">
         <is>
           <t>lag 27</t>
         </is>
       </c>
-      <c r="B30" s="48" t="n">
+      <c r="B30" s="47" t="n">
         <v>0.008004030604650998</v>
       </c>
-      <c r="C30" s="47" t="inlineStr">
+      <c r="C30" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D30" s="52" t="n">
+      <c r="D30" s="51" t="n">
         <v>0.008004030604650998</v>
       </c>
-      <c r="E30" s="50" t="inlineStr"/>
-      <c r="F30" s="51" t="inlineStr">
+      <c r="E30" s="49" t="inlineStr"/>
+      <c r="F30" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="A31" s="47" t="inlineStr">
+      <c r="A31" s="46" t="inlineStr">
         <is>
           <t>lag 28</t>
         </is>
       </c>
-      <c r="B31" s="48" t="n">
+      <c r="B31" s="47" t="n">
         <v>0.008589939238408145</v>
       </c>
-      <c r="C31" s="47" t="inlineStr">
+      <c r="C31" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D31" s="52" t="n">
+      <c r="D31" s="51" t="n">
         <v>0.008589939238408145</v>
       </c>
-      <c r="E31" s="50" t="inlineStr"/>
-      <c r="F31" s="51" t="inlineStr">
+      <c r="E31" s="49" t="inlineStr"/>
+      <c r="F31" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
-      <c r="A32" s="47" t="inlineStr">
+      <c r="A32" s="46" t="inlineStr">
         <is>
           <t>lag 29</t>
         </is>
       </c>
-      <c r="B32" s="48" t="n">
+      <c r="B32" s="47" t="n">
         <v>0.00795872626437487</v>
       </c>
-      <c r="C32" s="47" t="inlineStr">
+      <c r="C32" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D32" s="52" t="n">
+      <c r="D32" s="51" t="n">
         <v>0.00795872626437487</v>
       </c>
-      <c r="E32" s="50" t="inlineStr"/>
-      <c r="F32" s="51" t="inlineStr">
+      <c r="E32" s="49" t="inlineStr"/>
+      <c r="F32" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
-      <c r="A33" s="47" t="inlineStr">
+      <c r="A33" s="46" t="inlineStr">
         <is>
           <t>lag 30</t>
         </is>
       </c>
-      <c r="B33" s="48" t="n">
+      <c r="B33" s="47" t="n">
         <v>0.006683547200914103</v>
       </c>
-      <c r="C33" s="47" t="inlineStr">
+      <c r="C33" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D33" s="52" t="n">
+      <c r="D33" s="51" t="n">
         <v>0.006683547200914103</v>
       </c>
-      <c r="E33" s="50" t="inlineStr"/>
-      <c r="F33" s="51" t="inlineStr">
+      <c r="E33" s="49" t="inlineStr"/>
+      <c r="F33" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
-      <c r="A34" s="47" t="inlineStr">
+      <c r="A34" s="46" t="inlineStr">
         <is>
           <t>lag 31</t>
         </is>
       </c>
-      <c r="B34" s="48" t="n">
+      <c r="B34" s="47" t="n">
         <v>0.005250505593285775</v>
       </c>
-      <c r="C34" s="47" t="inlineStr">
+      <c r="C34" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D34" s="52" t="n">
+      <c r="D34" s="51" t="n">
         <v>0.005250505593285775</v>
       </c>
-      <c r="E34" s="50" t="inlineStr"/>
-      <c r="F34" s="51" t="inlineStr">
+      <c r="E34" s="49" t="inlineStr"/>
+      <c r="F34" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
-      <c r="A35" s="47" t="inlineStr">
+      <c r="A35" s="46" t="inlineStr">
         <is>
           <t>lag 32</t>
         </is>
       </c>
-      <c r="B35" s="48" t="n">
+      <c r="B35" s="47" t="n">
         <v>0.00568597289102907</v>
       </c>
-      <c r="C35" s="47" t="inlineStr">
+      <c r="C35" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D35" s="52" t="n">
+      <c r="D35" s="51" t="n">
         <v>0.00568597289102907</v>
       </c>
-      <c r="E35" s="50" t="inlineStr"/>
-      <c r="F35" s="51" t="inlineStr">
+      <c r="E35" s="49" t="inlineStr"/>
+      <c r="F35" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
-      <c r="A36" s="47" t="inlineStr">
+      <c r="A36" s="46" t="inlineStr">
         <is>
           <t>lag 33</t>
         </is>
       </c>
-      <c r="B36" s="48" t="n">
+      <c r="B36" s="47" t="n">
         <v>0.00221483942414175</v>
       </c>
-      <c r="C36" s="47" t="inlineStr">
+      <c r="C36" s="46" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D36" s="52" t="n">
+      <c r="D36" s="51" t="n">
         <v>0.00221483942414175</v>
       </c>
-      <c r="E36" s="50" t="inlineStr"/>
-      <c r="F36" s="51" t="inlineStr">
+      <c r="E36" s="49" t="inlineStr"/>
+      <c r="F36" s="50" t="inlineStr">
         <is>
           <t>full</t>
         </is>
@@ -16905,11 +19288,6 @@
           <t>Col E (Override): if filled, model uses it instead of auto value. Recent curve is preferred for lags 1-16; full curve covers longer lags from 2023 cohorts.</t>
         </is>
       </c>
-      <c r="B38" s="59" t="n"/>
-      <c r="C38" s="59" t="n"/>
-      <c r="D38" s="59" t="n"/>
-      <c r="E38" s="59" t="n"/>
-      <c r="F38" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -16942,9 +19320,6 @@
           <t>Flat Prolongation Rate by Dim  —  EDIT yellow column  (fallback when no payment_no data)</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="59" t="n"/>
-      <c r="D1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -16969,7 +19344,7 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="42" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>Base/Private</t>
         </is>
@@ -16977,17 +19352,17 @@
       <c r="B3" s="18" t="n">
         <v>0.458</v>
       </c>
-      <c r="C3" s="53" t="n">
+      <c r="C3" s="52" t="n">
         <v>0.458</v>
       </c>
-      <c r="D3" s="54" t="inlineStr">
+      <c r="D3" s="53" t="inlineStr">
         <is>
           <t>data pool=1655 sec=758</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Base/Premium</t>
         </is>
@@ -16995,17 +19370,17 @@
       <c r="B4" s="18" t="n">
         <v>0.3654</v>
       </c>
-      <c r="C4" s="53" t="n">
+      <c r="C4" s="52" t="n">
         <v>0.3654</v>
       </c>
-      <c r="D4" s="54" t="inlineStr">
+      <c r="D4" s="53" t="inlineStr">
         <is>
           <t>data pool=1853 sec=677</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>Base/Group</t>
         </is>
@@ -17013,17 +19388,17 @@
       <c r="B5" s="18" t="n">
         <v>0.4462</v>
       </c>
-      <c r="C5" s="53" t="n">
+      <c r="C5" s="52" t="n">
         <v>0.4462</v>
       </c>
-      <c r="D5" s="54" t="inlineStr">
+      <c r="D5" s="53" t="inlineStr">
         <is>
           <t>data pool=7645 sec=3411</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="55" t="inlineStr">
+      <c r="A6" s="54" t="inlineStr">
         <is>
           <t>MT/Private</t>
         </is>
@@ -17031,17 +19406,17 @@
       <c r="B6" s="18" t="n">
         <v>0.6591</v>
       </c>
-      <c r="C6" s="53" t="n">
+      <c r="C6" s="52" t="n">
         <v>0.6591</v>
       </c>
-      <c r="D6" s="54" t="inlineStr">
+      <c r="D6" s="53" t="inlineStr">
         <is>
           <t>data pool=88 sec=58</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="45" t="inlineStr">
+      <c r="A7" s="44" t="inlineStr">
         <is>
           <t>MT/Premium</t>
         </is>
@@ -17049,10 +19424,10 @@
       <c r="B7" s="18" t="n">
         <v>0.435</v>
       </c>
-      <c r="C7" s="53" t="n">
+      <c r="C7" s="52" t="n">
         <v>0.435</v>
       </c>
-      <c r="D7" s="54" t="inlineStr">
+      <c r="D7" s="53" t="inlineStr">
         <is>
           <t>hardcoded default (pool=3&lt;15)</t>
         </is>
@@ -17067,10 +19442,10 @@
       <c r="B8" s="18" t="n">
         <v>0.435</v>
       </c>
-      <c r="C8" s="53" t="n">
+      <c r="C8" s="52" t="n">
         <v>0.435</v>
       </c>
-      <c r="D8" s="54" t="inlineStr">
+      <c r="D8" s="53" t="inlineStr">
         <is>
           <t>hardcoded default (pool=7&lt;15)</t>
         </is>
@@ -17082,9 +19457,6 @@
           <t>Global fallback rate (when pool &lt; 15): 0.4345  (pool=11376, sec=4943)</t>
         </is>
       </c>
-      <c r="B9" s="59" t="n"/>
-      <c r="C9" s="59" t="n"/>
-      <c r="D9" s="60" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
@@ -17092,9 +19464,6 @@
           <t>This flat rate is used as a fallback in mode=ext (Jun-Dec 2026) for pool_display calculation. For mode=data/blend the model uses retention_by_renewal[pno] instead.</t>
         </is>
       </c>
-      <c r="B11" s="59" t="n"/>
-      <c r="C11" s="59" t="n"/>
-      <c r="D11" s="60" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -17126,8 +19495,6 @@
           <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
         </is>
       </c>
-      <c r="B1" s="59" t="n"/>
-      <c r="C1" s="60" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -17147,13 +19514,11 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="56" t="inlineStr">
+      <c r="A3" s="55" t="inlineStr">
         <is>
           <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
         </is>
       </c>
-      <c r="B3" s="59" t="n"/>
-      <c r="C3" s="60" t="n"/>
     </row>
     <row r="4" ht="47" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -17161,7 +19526,7 @@
           <t>data_cutoff</t>
         </is>
       </c>
-      <c r="B4" s="57" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
@@ -17178,7 +19543,7 @@
           <t>cal_window_start</t>
         </is>
       </c>
-      <c r="B5" s="57" t="inlineStr">
+      <c r="B5" s="56" t="inlineStr">
         <is>
           <t>2025-07</t>
         </is>
@@ -17195,7 +19560,7 @@
           <t>cal_window_end</t>
         </is>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="56" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
@@ -17212,7 +19577,7 @@
           <t>forecast_start</t>
         </is>
       </c>
-      <c r="B7" s="57" t="inlineStr">
+      <c r="B7" s="56" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
@@ -17229,7 +19594,7 @@
           <t>forecast_end</t>
         </is>
       </c>
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="56" t="inlineStr">
         <is>
           <t>2026-12</t>
         </is>
@@ -17241,13 +19606,11 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="56" t="inlineStr">
+      <c r="A9" s="55" t="inlineStr">
         <is>
           <t>── КОРРЕКЦИЯ AOV ──</t>
         </is>
       </c>
-      <c r="B9" s="59" t="n"/>
-      <c r="C9" s="60" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -17255,7 +19618,7 @@
           <t>aov_adjustment_factor</t>
         </is>
       </c>
-      <c r="B10" s="58" t="n">
+      <c r="B10" s="57" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="30" t="inlineStr">
@@ -17270,13 +19633,11 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="56" t="inlineStr">
+      <c r="A11" s="55" t="inlineStr">
         <is>
           <t>── РОСТ ЦЕН ──</t>
         </is>
       </c>
-      <c r="B11" s="59" t="n"/>
-      <c r="C11" s="60" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -17284,7 +19645,7 @@
           <t>price_growth_pct_per_quarter</t>
         </is>
       </c>
-      <c r="B12" s="58" t="n">
+      <c r="B12" s="57" t="n">
         <v>0.03</v>
       </c>
       <c r="C12" s="30" t="inlineStr">
@@ -17299,7 +19660,7 @@
           <t>price_base_year</t>
         </is>
       </c>
-      <c r="B13" s="57" t="n">
+      <c r="B13" s="56" t="n">
         <v>2025</v>
       </c>
       <c r="C13" s="30" t="inlineStr">
@@ -17314,7 +19675,7 @@
           <t>price_base_quarter</t>
         </is>
       </c>
-      <c r="B14" s="57" t="n">
+      <c r="B14" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="30" t="inlineStr">
@@ -17324,13 +19685,11 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="56" t="inlineStr">
+      <c r="A15" s="55" t="inlineStr">
         <is>
           <t>── КОРРЕКТИРОВКА RETENTION ──</t>
         </is>
       </c>
-      <c r="B15" s="59" t="n"/>
-      <c r="C15" s="60" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
@@ -17338,7 +19697,7 @@
           <t>retention_adjustment</t>
         </is>
       </c>
-      <c r="B16" s="58" t="n">
+      <c r="B16" s="57" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Implement three-pool retention model: pool[T] + pool[T+1] + pool[T-1]
Secondary sales in month T come from three sources:
  pool[T]   × rate_present  - students paying on time
  pool[T+1] × rate_earlier  - students paying early (dosrochnye)
  pool[T-1] × rate_reanim   - students paying late (zazdershavshiesya)

Calibrated rates:
  pno=1: present=14.9%, earlier=7.3%, reanim=3.2%
  pno=5: present=42.3%, earlier=17.1%, reanim=6.6%

Segment shares NOW affect N (not just AOV):
  Changing Earlier from 31% to 44% → earlier×1.43 scaling
  → pool[T+1] contribution +43% → timing shift forward

Excel: retention_by_renewal sheet now has THREE-POOL RATES section
  pno | rate_present | rate_earlier_1 | rate_reanim_1 (all editable)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -190,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -212,11 +212,55 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -338,6 +382,9 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -380,15 +427,14 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -993,6 +1039,19 @@
           <t>Primary Student Plan Counts (Jan-Dec 2026)  —  EDIT yellow cells</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+      <c r="F1" s="58" t="n"/>
+      <c r="G1" s="58" t="n"/>
+      <c r="H1" s="58" t="n"/>
+      <c r="I1" s="58" t="n"/>
+      <c r="J1" s="58" t="n"/>
+      <c r="K1" s="58" t="n"/>
+      <c r="L1" s="58" t="n"/>
+      <c r="M1" s="58" t="n"/>
+      <c r="N1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -1394,6 +1453,19 @@
           <t>Edit yellow cells to change the primary student plan, then re-run forecast_2026_v3.py</t>
         </is>
       </c>
+      <c r="B11" s="58" t="n"/>
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="58" t="n"/>
+      <c r="I11" s="58" t="n"/>
+      <c r="J11" s="58" t="n"/>
+      <c r="K11" s="58" t="n"/>
+      <c r="L11" s="58" t="n"/>
+      <c r="M11" s="58" t="n"/>
+      <c r="N11" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1425,6 +1497,9 @@
           <t>Package Distribution  —  secondary sales Jul-Dec 2025  |  EDIT yellow cells to override</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -7430,6 +7505,9 @@
           <t>Probabilities are auto-normalized per dim in the model. Edit to override distribution.</t>
         </is>
       </c>
+      <c r="B336" s="58" t="n"/>
+      <c r="C336" s="58" t="n"/>
+      <c r="D336" s="59" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="30" t="inlineStr">
@@ -7437,6 +7515,9 @@
           <t>MT dims with thin data use Base/{}-fallback. Base/Group hardcoded fallback: {8: 0.25, 10: 0.14, 32: 0.13, 16: 0.13, 20: 0.09, 4: 0.08, 36: 0.07, 40: 0.06}</t>
         </is>
       </c>
+      <c r="B337" s="58" t="n"/>
+      <c r="C337" s="58" t="n"/>
+      <c r="D337" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7471,6 +7552,11 @@
           <t>Renewal Price per Lesson (base Q3-2025)  —  EDIT yellow cells to override</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+      <c r="F1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15478,6 +15564,11 @@
           <t>Base period: Q3-2025 (Jul-Sep). Growth factor = (1+3%)^(quarters from Q3-2025). Jan-2026 is Q1-2026 = 2 quarters after Q3-2025, so pgf = 1.0609.</t>
         </is>
       </c>
+      <c r="B336" s="58" t="n"/>
+      <c r="C336" s="58" t="n"/>
+      <c r="D336" s="58" t="n"/>
+      <c r="E336" s="58" t="n"/>
+      <c r="F336" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15494,7 +15585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -15513,6 +15604,13 @@
           <t>Retention by (pno, ct, gt, pkg_bucket)  —  Override column takes priority. Fallback: pkg_bucket=ALL (dim-level), then global pno default.</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+      <c r="F1" s="58" t="n"/>
+      <c r="G1" s="58" t="n"/>
+      <c r="H1" s="59" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -15520,6 +15618,13 @@
           <t>Fallback hierarchy: Level1=(pno,ct,gt,pkg) pool&gt;=15  →  Level2=(pno,ct,gt) ALL  →  Level3=global(pno)</t>
         </is>
       </c>
+      <c r="B2" s="58" t="n"/>
+      <c r="C2" s="58" t="n"/>
+      <c r="D2" s="58" t="n"/>
+      <c r="E2" s="58" t="n"/>
+      <c r="F2" s="58" t="n"/>
+      <c r="G2" s="58" t="n"/>
+      <c r="H2" s="59" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -18331,11 +18436,532 @@
           <t>pno=1 = primary (not secondary). pno=2 = first renewal. Override (col F) takes priority over Retention (col E) if non-empty. pkg_bucket rows = Level-1 (pool&gt;=15). ALL rows = Level-2 fallback. For pno&gt;=16 model uses RETENTION_PNO_HIGH=72.0%.</t>
         </is>
       </c>
+      <c r="B96" s="58" t="n"/>
+      <c r="C96" s="58" t="n"/>
+      <c r="D96" s="58" t="n"/>
+      <c r="E96" s="58" t="n"/>
+      <c r="F96" s="58" t="n"/>
+      <c r="G96" s="58" t="n"/>
+      <c r="H96" s="59" t="n"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="41" t="inlineStr">
+        <is>
+          <t>━━━━━━━━  THREE-POOL RATES  ━━━━━━━━  Hist shares: Present=0.497  Earlier=0.310  Reanim=0.108  —  Edit rates below; scaling applied by forecast_2026_v3.py based on shares sheet</t>
+        </is>
+      </c>
+      <c r="B98" s="58" t="n"/>
+      <c r="C98" s="58" t="n"/>
+      <c r="D98" s="58" t="n"/>
+      <c r="E98" s="58" t="n"/>
+      <c r="F98" s="58" t="n"/>
+      <c r="G98" s="58" t="n"/>
+      <c r="H98" s="59" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>pno</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>rate_present</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>rate_earlier_1</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>rate_reanim_1</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="inlineStr">
+        <is>
+          <t>note_present</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="inlineStr">
+        <is>
+          <t>note_earlier</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>note_reanim</t>
+        </is>
+      </c>
+      <c r="H99" s="9" t="inlineStr">
+        <is>
+          <t>hist_shares</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B100" s="18" t="n">
+        <v>0.1494</v>
+      </c>
+      <c r="C100" s="18" t="n">
+        <v>0.0727</v>
+      </c>
+      <c r="D100" s="18" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="E100" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=6648 sec=993</t>
+        </is>
+      </c>
+      <c r="F100" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=5721 sec=416</t>
+        </is>
+      </c>
+      <c r="G100" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=5514 sec=174</t>
+        </is>
+      </c>
+      <c r="H100" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B101" s="18" t="n">
+        <v>0.2636</v>
+      </c>
+      <c r="C101" s="18" t="n">
+        <v>0.1394</v>
+      </c>
+      <c r="D101" s="18" t="n">
+        <v>0.0546</v>
+      </c>
+      <c r="E101" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=2432 sec=641</t>
+        </is>
+      </c>
+      <c r="F101" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=2059 sec=287</t>
+        </is>
+      </c>
+      <c r="G101" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=2032 sec=111</t>
+        </is>
+      </c>
+      <c r="H101" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B102" s="18" t="n">
+        <v>0.3097</v>
+      </c>
+      <c r="C102" s="18" t="n">
+        <v>0.1633</v>
+      </c>
+      <c r="D102" s="18" t="n">
+        <v>0.07770000000000001</v>
+      </c>
+      <c r="E102" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=972 sec=301</t>
+        </is>
+      </c>
+      <c r="F102" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=833 sec=136</t>
+        </is>
+      </c>
+      <c r="G102" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=824 sec=64</t>
+        </is>
+      </c>
+      <c r="H102" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B103" s="18" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="C103" s="18" t="n">
+        <v>0.2141</v>
+      </c>
+      <c r="D103" s="18" t="n">
+        <v>0.0694</v>
+      </c>
+      <c r="E103" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=535 sec=168</t>
+        </is>
+      </c>
+      <c r="F103" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=439 sec=94</t>
+        </is>
+      </c>
+      <c r="G103" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=447 sec=31</t>
+        </is>
+      </c>
+      <c r="H103" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B104" s="18" t="n">
+        <v>0.4225</v>
+      </c>
+      <c r="C104" s="18" t="n">
+        <v>0.1944</v>
+      </c>
+      <c r="D104" s="18" t="n">
+        <v>0.07489999999999999</v>
+      </c>
+      <c r="E104" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=258 sec=109</t>
+        </is>
+      </c>
+      <c r="F104" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=216 sec=42</t>
+        </is>
+      </c>
+      <c r="G104" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=227 sec=17</t>
+        </is>
+      </c>
+      <c r="H104" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B105" s="18" t="n">
+        <v>0.3989</v>
+      </c>
+      <c r="C105" s="18" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D105" s="18" t="n">
+        <v>0.1133</v>
+      </c>
+      <c r="E105" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=178 sec=71</t>
+        </is>
+      </c>
+      <c r="F105" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=150 sec=36</t>
+        </is>
+      </c>
+      <c r="G105" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=150 sec=17</t>
+        </is>
+      </c>
+      <c r="H105" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B106" s="18" t="n">
+        <v>0.4495</v>
+      </c>
+      <c r="C106" s="18" t="n">
+        <v>0.2391</v>
+      </c>
+      <c r="D106" s="18" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="E106" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=109 sec=49</t>
+        </is>
+      </c>
+      <c r="F106" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=92 sec=22</t>
+        </is>
+      </c>
+      <c r="G106" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=92 sec=8</t>
+        </is>
+      </c>
+      <c r="H106" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B107" s="18" t="n">
+        <v>0.5155999999999999</v>
+      </c>
+      <c r="C107" s="18" t="n">
+        <v>0.07140000000000001</v>
+      </c>
+      <c r="D107" s="18" t="n">
+        <v>0.1481</v>
+      </c>
+      <c r="E107" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=64 sec=33</t>
+        </is>
+      </c>
+      <c r="F107" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=56 sec=4</t>
+        </is>
+      </c>
+      <c r="G107" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=54 sec=8</t>
+        </is>
+      </c>
+      <c r="H107" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" s="37" t="n">
+        <v>9</v>
+      </c>
+      <c r="B108" s="18" t="n">
+        <v>0.6383</v>
+      </c>
+      <c r="C108" s="18" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="D108" s="18" t="n">
+        <v>0.07140000000000001</v>
+      </c>
+      <c r="E108" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=47 sec=30</t>
+        </is>
+      </c>
+      <c r="F108" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=36 sec=4</t>
+        </is>
+      </c>
+      <c r="G108" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=42 sec=3</t>
+        </is>
+      </c>
+      <c r="H108" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="B109" s="18" t="n">
+        <v>0.6111</v>
+      </c>
+      <c r="C109" s="18" t="n">
+        <v>0.0312</v>
+      </c>
+      <c r="D109" s="18" t="n">
+        <v>0.1724</v>
+      </c>
+      <c r="E109" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=36 sec=22</t>
+        </is>
+      </c>
+      <c r="F109" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=32 sec=1</t>
+        </is>
+      </c>
+      <c r="G109" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=29 sec=5</t>
+        </is>
+      </c>
+      <c r="H109" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1">
+      <c r="A110" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="B110" s="18" t="n">
+        <v>0.5758</v>
+      </c>
+      <c r="C110" s="18" t="n">
+        <v>0.1739</v>
+      </c>
+      <c r="D110" s="18" t="n">
+        <v>0.1333</v>
+      </c>
+      <c r="E110" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=33 sec=19</t>
+        </is>
+      </c>
+      <c r="F110" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=23 sec=4</t>
+        </is>
+      </c>
+      <c r="G110" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=30 sec=4</t>
+        </is>
+      </c>
+      <c r="H110" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" s="37" t="n">
+        <v>12</v>
+      </c>
+      <c r="B111" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C111" s="18" t="n">
+        <v>0.1765</v>
+      </c>
+      <c r="D111" s="18" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="E111" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=20 sec=10</t>
+        </is>
+      </c>
+      <c r="F111" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=17 sec=3</t>
+        </is>
+      </c>
+      <c r="G111" s="19" t="inlineStr">
+        <is>
+          <t>data pool_Tm1=18 sec=2</t>
+        </is>
+      </c>
+      <c r="H111" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1">
+      <c r="A112" s="37" t="n">
+        <v>13</v>
+      </c>
+      <c r="B112" s="18" t="n">
+        <v>0.4545</v>
+      </c>
+      <c r="C112" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D112" s="18" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E112" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T=11 sec=5</t>
+        </is>
+      </c>
+      <c r="F112" s="19" t="inlineStr">
+        <is>
+          <t>data pool_T1=10 sec=2</t>
+        </is>
+      </c>
+      <c r="G112" s="19" t="inlineStr">
+        <is>
+          <t>hardcoded default (pool_Tm1=9&lt;10)</t>
+        </is>
+      </c>
+      <c r="H112" s="19" t="inlineStr">
+        <is>
+          <t>Present_hist=0.497  Earlier_hist=0.31  Reanim_hist=0.108</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="30" t="inlineStr">
+        <is>
+          <t>THREE-POOL section is read by forecast_2026_v3.py for data/blend mode months. rate_present = pool[T]×rate→sec; rate_earlier = pool[T+1]×rate→early-pay; rate_reanim = pool[T-1]×rate→late-pay. Effective rates are scaled by (current_share / hist_share) from the shares sheet.</t>
+        </is>
+      </c>
+      <c r="B114" s="58" t="n"/>
+      <c r="C114" s="58" t="n"/>
+      <c r="D114" s="58" t="n"/>
+      <c r="E114" s="58" t="n"/>
+      <c r="F114" s="58" t="n"/>
+      <c r="G114" s="58" t="n"/>
+      <c r="H114" s="59" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
+    <mergeCell ref="A114:H114"/>
     <mergeCell ref="A96:H96"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A98:H98"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18362,6 +18988,8 @@
           <t>Segment Shares  —  EDIT yellow column (must sum to 1.0 across all 4 segments)</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -18381,14 +19009,12 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n">
-        <v>0.4971</v>
-      </c>
+      <c r="B3" s="18" t="n"/>
       <c r="C3" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid in expected month (paid_M == prev_plan_M)</t>
@@ -18396,14 +19022,12 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Earlier</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
-        <v>0.3103</v>
-      </c>
+      <c r="B4" s="18" t="n"/>
       <c r="C4" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid before expected month (paid_M &lt; prev_plan_M)</t>
@@ -18411,14 +19035,12 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>Reanim</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>0.1078</v>
-      </c>
+      <c r="B5" s="18" t="n"/>
       <c r="C5" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid after expected month (paid_M &gt; prev_plan_M)</t>
@@ -18426,14 +19048,12 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="45" t="inlineStr">
         <is>
           <t>Upgrades</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
-        <v>0.0848</v>
-      </c>
+      <c r="B6" s="18" t="n"/>
       <c r="C6" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | cat_payment = secondary upgrade</t>
@@ -18446,7 +19066,7 @@
           <t>SUM</t>
         </is>
       </c>
-      <c r="B7" s="45" t="n">
+      <c r="B7" s="46" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="28" t="inlineStr">
@@ -18455,12 +19075,15 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Edit yellow cells. The model normalizes shares automatically if sum != 1.0.</t>
         </is>
       </c>
+      <c r="B9" s="58" t="n"/>
+      <c r="C9" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -18494,6 +19117,11 @@
           <t>Ext-curve (Lag Curve for Future Cohorts)  —  EDIT col E (Override) only if needed</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="58" t="n"/>
+      <c r="E1" s="58" t="n"/>
+      <c r="F1" s="59" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -18501,6 +19129,11 @@
           <t>Recent (2024-01 to 2025-06): lags 1-22  |  Full fallback (2023-01 to 2025-06): lags 23-33  |  Used by mode=ext (Jun-Dec 2026)</t>
         </is>
       </c>
+      <c r="B2" s="58" t="n"/>
+      <c r="C2" s="58" t="n"/>
+      <c r="D2" s="58" t="n"/>
+      <c r="E2" s="58" t="n"/>
+      <c r="F2" s="59" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -18535,748 +19168,748 @@
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>lag 1</t>
         </is>
       </c>
-      <c r="B4" s="47" t="n">
+      <c r="B4" s="48" t="n">
         <v>0.03243981260767305</v>
       </c>
-      <c r="C4" s="47" t="n">
+      <c r="C4" s="48" t="n">
         <v>0.03325380378132611</v>
       </c>
-      <c r="D4" s="48" t="n">
+      <c r="D4" s="49" t="n">
         <v>0.03325380378132611</v>
       </c>
-      <c r="E4" s="49" t="inlineStr"/>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="E4" s="50" t="inlineStr"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>lag 2</t>
         </is>
       </c>
-      <c r="B5" s="47" t="n">
+      <c r="B5" s="48" t="n">
         <v>0.05565081335823394</v>
       </c>
-      <c r="C5" s="47" t="n">
+      <c r="C5" s="48" t="n">
         <v>0.05229594677145271</v>
       </c>
-      <c r="D5" s="48" t="n">
+      <c r="D5" s="49" t="n">
         <v>0.05229594677145271</v>
       </c>
-      <c r="E5" s="49" t="inlineStr"/>
-      <c r="F5" s="50" t="inlineStr">
+      <c r="E5" s="50" t="inlineStr"/>
+      <c r="F5" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>lag 3</t>
         </is>
       </c>
-      <c r="B6" s="47" t="n">
+      <c r="B6" s="48" t="n">
         <v>0.05740292312901271</v>
       </c>
-      <c r="C6" s="47" t="n">
+      <c r="C6" s="48" t="n">
         <v>0.04043051008979147</v>
       </c>
-      <c r="D6" s="48" t="n">
+      <c r="D6" s="49" t="n">
         <v>0.04043051008979147</v>
       </c>
-      <c r="E6" s="49" t="inlineStr"/>
-      <c r="F6" s="50" t="inlineStr">
+      <c r="E6" s="50" t="inlineStr"/>
+      <c r="F6" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>lag 4</t>
         </is>
       </c>
-      <c r="B7" s="47" t="n">
+      <c r="B7" s="48" t="n">
         <v>0.08721467251692649</v>
       </c>
-      <c r="C7" s="47" t="n">
+      <c r="C7" s="48" t="n">
         <v>0.06933519380542201</v>
       </c>
-      <c r="D7" s="48" t="n">
+      <c r="D7" s="49" t="n">
         <v>0.06933519380542201</v>
       </c>
-      <c r="E7" s="49" t="inlineStr"/>
-      <c r="F7" s="50" t="inlineStr">
+      <c r="E7" s="50" t="inlineStr"/>
+      <c r="F7" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="8" ht="14" customHeight="1">
-      <c r="A8" s="46" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>lag 5</t>
         </is>
       </c>
-      <c r="B8" s="47" t="n">
+      <c r="B8" s="48" t="n">
         <v>0.04908093490622328</v>
       </c>
-      <c r="C8" s="47" t="n">
+      <c r="C8" s="48" t="n">
         <v>0.04150558638908253</v>
       </c>
-      <c r="D8" s="48" t="n">
+      <c r="D8" s="49" t="n">
         <v>0.04150558638908253</v>
       </c>
-      <c r="E8" s="49" t="inlineStr"/>
-      <c r="F8" s="50" t="inlineStr">
+      <c r="E8" s="50" t="inlineStr"/>
+      <c r="F8" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="9" ht="14" customHeight="1">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>lag 6</t>
         </is>
       </c>
-      <c r="B9" s="47" t="n">
+      <c r="B9" s="48" t="n">
         <v>0.04107542987799979</v>
       </c>
-      <c r="C9" s="47" t="n">
+      <c r="C9" s="48" t="n">
         <v>0.03334841325604449</v>
       </c>
-      <c r="D9" s="48" t="n">
+      <c r="D9" s="49" t="n">
         <v>0.03334841325604449</v>
       </c>
-      <c r="E9" s="49" t="inlineStr"/>
-      <c r="F9" s="50" t="inlineStr">
+      <c r="E9" s="50" t="inlineStr"/>
+      <c r="F9" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14" customHeight="1">
-      <c r="A10" s="46" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>lag 7</t>
         </is>
       </c>
-      <c r="B10" s="47" t="n">
+      <c r="B10" s="48" t="n">
         <v>0.04132556188857849</v>
       </c>
-      <c r="C10" s="47" t="n">
+      <c r="C10" s="48" t="n">
         <v>0.04115337003794277</v>
       </c>
-      <c r="D10" s="48" t="n">
+      <c r="D10" s="49" t="n">
         <v>0.04115337003794277</v>
       </c>
-      <c r="E10" s="49" t="inlineStr"/>
-      <c r="F10" s="50" t="inlineStr">
+      <c r="E10" s="50" t="inlineStr"/>
+      <c r="F10" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>lag 8</t>
         </is>
       </c>
-      <c r="B11" s="47" t="n">
+      <c r="B11" s="48" t="n">
         <v>0.07794682286006098</v>
       </c>
-      <c r="C11" s="47" t="n">
+      <c r="C11" s="48" t="n">
         <v>0.08012093056296371</v>
       </c>
-      <c r="D11" s="48" t="n">
+      <c r="D11" s="49" t="n">
         <v>0.08012093056296371</v>
       </c>
-      <c r="E11" s="49" t="inlineStr"/>
-      <c r="F11" s="50" t="inlineStr">
+      <c r="E11" s="50" t="inlineStr"/>
+      <c r="F11" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="12" ht="14" customHeight="1">
-      <c r="A12" s="46" t="inlineStr">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>lag 9</t>
         </is>
       </c>
-      <c r="B12" s="47" t="n">
+      <c r="B12" s="48" t="n">
         <v>0.05219903571086893</v>
       </c>
-      <c r="C12" s="47" t="n">
+      <c r="C12" s="48" t="n">
         <v>0.0463728113540315</v>
       </c>
-      <c r="D12" s="48" t="n">
+      <c r="D12" s="49" t="n">
         <v>0.0463728113540315</v>
       </c>
-      <c r="E12" s="49" t="inlineStr"/>
-      <c r="F12" s="50" t="inlineStr">
+      <c r="E12" s="50" t="inlineStr"/>
+      <c r="F12" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>lag 10</t>
         </is>
       </c>
-      <c r="B13" s="47" t="n">
+      <c r="B13" s="48" t="n">
         <v>0.0263084995491605</v>
       </c>
-      <c r="C13" s="47" t="n">
+      <c r="C13" s="48" t="n">
         <v>0.02540345997477899</v>
       </c>
-      <c r="D13" s="48" t="n">
+      <c r="D13" s="49" t="n">
         <v>0.02540345997477899</v>
       </c>
-      <c r="E13" s="49" t="inlineStr"/>
-      <c r="F13" s="50" t="inlineStr">
+      <c r="E13" s="50" t="inlineStr"/>
+      <c r="F13" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14" customHeight="1">
-      <c r="A14" s="46" t="inlineStr">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>lag 11</t>
         </is>
       </c>
-      <c r="B14" s="47" t="n">
+      <c r="B14" s="48" t="n">
         <v>0.01694534590044715</v>
       </c>
-      <c r="C14" s="47" t="n">
+      <c r="C14" s="48" t="n">
         <v>0.01670792262887267</v>
       </c>
-      <c r="D14" s="48" t="n">
+      <c r="D14" s="49" t="n">
         <v>0.01670792262887267</v>
       </c>
-      <c r="E14" s="49" t="inlineStr"/>
-      <c r="F14" s="50" t="inlineStr">
+      <c r="E14" s="50" t="inlineStr"/>
+      <c r="F14" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14" customHeight="1">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>lag 12</t>
         </is>
       </c>
-      <c r="B15" s="47" t="n">
+      <c r="B15" s="48" t="n">
         <v>0.02311776204827275</v>
       </c>
-      <c r="C15" s="47" t="n">
+      <c r="C15" s="48" t="n">
         <v>0.0203014383813916</v>
       </c>
-      <c r="D15" s="48" t="n">
+      <c r="D15" s="49" t="n">
         <v>0.0203014383813916</v>
       </c>
-      <c r="E15" s="49" t="inlineStr"/>
-      <c r="F15" s="50" t="inlineStr">
+      <c r="E15" s="50" t="inlineStr"/>
+      <c r="F15" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="16" ht="14" customHeight="1">
-      <c r="A16" s="46" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>lag 13</t>
         </is>
       </c>
-      <c r="B16" s="47" t="n">
+      <c r="B16" s="48" t="n">
         <v>0.02009059602064579</v>
       </c>
-      <c r="C16" s="47" t="n">
+      <c r="C16" s="48" t="n">
         <v>0.0129558204440133</v>
       </c>
-      <c r="D16" s="48" t="n">
+      <c r="D16" s="49" t="n">
         <v>0.0129558204440133</v>
       </c>
-      <c r="E16" s="49" t="inlineStr"/>
-      <c r="F16" s="50" t="inlineStr">
+      <c r="E16" s="50" t="inlineStr"/>
+      <c r="F16" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="17" ht="14" customHeight="1">
-      <c r="A17" s="46" t="inlineStr">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>lag 14</t>
         </is>
       </c>
-      <c r="B17" s="47" t="n">
+      <c r="B17" s="48" t="n">
         <v>0.01442047607706917</v>
       </c>
-      <c r="C17" s="47" t="n">
+      <c r="C17" s="48" t="n">
         <v>0.0123686957085169</v>
       </c>
-      <c r="D17" s="48" t="n">
+      <c r="D17" s="49" t="n">
         <v>0.0123686957085169</v>
       </c>
-      <c r="E17" s="49" t="inlineStr"/>
-      <c r="F17" s="50" t="inlineStr">
+      <c r="E17" s="50" t="inlineStr"/>
+      <c r="F17" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="18" ht="14" customHeight="1">
-      <c r="A18" s="46" t="inlineStr">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>lag 15</t>
         </is>
       </c>
-      <c r="B18" s="47" t="n">
+      <c r="B18" s="48" t="n">
         <v>0.0190650878142931</v>
       </c>
-      <c r="C18" s="47" t="n">
+      <c r="C18" s="48" t="n">
         <v>0.02177364537386275</v>
       </c>
-      <c r="D18" s="48" t="n">
+      <c r="D18" s="49" t="n">
         <v>0.02177364537386275</v>
       </c>
-      <c r="E18" s="49" t="inlineStr"/>
-      <c r="F18" s="50" t="inlineStr">
+      <c r="E18" s="50" t="inlineStr"/>
+      <c r="F18" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14" customHeight="1">
-      <c r="A19" s="46" t="inlineStr">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>lag 16</t>
         </is>
       </c>
-      <c r="B19" s="47" t="n">
+      <c r="B19" s="48" t="n">
         <v>0.03493600983148009</v>
       </c>
-      <c r="C19" s="47" t="n">
+      <c r="C19" s="48" t="n">
         <v>0.03563806584503205</v>
       </c>
-      <c r="D19" s="48" t="n">
+      <c r="D19" s="49" t="n">
         <v>0.03563806584503205</v>
       </c>
-      <c r="E19" s="49" t="inlineStr"/>
-      <c r="F19" s="50" t="inlineStr">
+      <c r="E19" s="50" t="inlineStr"/>
+      <c r="F19" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14" customHeight="1">
-      <c r="A20" s="46" t="inlineStr">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>lag 17</t>
         </is>
       </c>
-      <c r="B20" s="47" t="n">
+      <c r="B20" s="48" t="n">
         <v>0.0265347588824575</v>
       </c>
-      <c r="C20" s="47" t="n">
+      <c r="C20" s="48" t="n">
         <v>0.02582494976486335</v>
       </c>
-      <c r="D20" s="48" t="n">
+      <c r="D20" s="49" t="n">
         <v>0.02582494976486335</v>
       </c>
-      <c r="E20" s="49" t="inlineStr"/>
-      <c r="F20" s="50" t="inlineStr">
+      <c r="E20" s="50" t="inlineStr"/>
+      <c r="F20" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="21" ht="14" customHeight="1">
-      <c r="A21" s="46" t="inlineStr">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>lag 18</t>
         </is>
       </c>
-      <c r="B21" s="47" t="n">
+      <c r="B21" s="48" t="n">
         <v>0.01720805529257647</v>
       </c>
-      <c r="C21" s="47" t="n">
+      <c r="C21" s="48" t="n">
         <v>0.0141590908625448</v>
       </c>
-      <c r="D21" s="48" t="n">
+      <c r="D21" s="49" t="n">
         <v>0.0141590908625448</v>
       </c>
-      <c r="E21" s="49" t="inlineStr"/>
-      <c r="F21" s="50" t="inlineStr">
+      <c r="E21" s="50" t="inlineStr"/>
+      <c r="F21" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
-      <c r="A22" s="46" t="inlineStr">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>lag 19</t>
         </is>
       </c>
-      <c r="B22" s="47" t="n">
+      <c r="B22" s="48" t="n">
         <v>0.01112484167561391</v>
       </c>
-      <c r="C22" s="47" t="n">
+      <c r="C22" s="48" t="n">
         <v>0.01008889509869752</v>
       </c>
-      <c r="D22" s="48" t="n">
+      <c r="D22" s="49" t="n">
         <v>0.01008889509869752</v>
       </c>
-      <c r="E22" s="49" t="inlineStr"/>
-      <c r="F22" s="50" t="inlineStr">
+      <c r="E22" s="50" t="inlineStr"/>
+      <c r="F22" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="23" ht="14" customHeight="1">
-      <c r="A23" s="46" t="inlineStr">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>lag 20</t>
         </is>
       </c>
-      <c r="B23" s="47" t="n">
+      <c r="B23" s="48" t="n">
         <v>0.01020671444500314</v>
       </c>
-      <c r="C23" s="47" t="n">
+      <c r="C23" s="48" t="n">
         <v>0.009296585755124544</v>
       </c>
-      <c r="D23" s="48" t="n">
+      <c r="D23" s="49" t="n">
         <v>0.009296585755124544</v>
       </c>
-      <c r="E23" s="49" t="inlineStr"/>
-      <c r="F23" s="50" t="inlineStr">
+      <c r="E23" s="50" t="inlineStr"/>
+      <c r="F23" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="24" ht="14" customHeight="1">
-      <c r="A24" s="46" t="inlineStr">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>lag 21</t>
         </is>
       </c>
-      <c r="B24" s="47" t="n">
+      <c r="B24" s="48" t="n">
         <v>0.009025071771145076</v>
       </c>
-      <c r="C24" s="47" t="n">
+      <c r="C24" s="48" t="n">
         <v>0.00748335033616986</v>
       </c>
-      <c r="D24" s="48" t="n">
+      <c r="D24" s="49" t="n">
         <v>0.00748335033616986</v>
       </c>
-      <c r="E24" s="49" t="inlineStr"/>
-      <c r="F24" s="50" t="inlineStr">
+      <c r="E24" s="50" t="inlineStr"/>
+      <c r="F24" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
-      <c r="A25" s="46" t="inlineStr">
+      <c r="A25" s="47" t="inlineStr">
         <is>
           <t>lag 22</t>
         </is>
       </c>
-      <c r="B25" s="47" t="n">
+      <c r="B25" s="48" t="n">
         <v>0.01282232984589626</v>
       </c>
-      <c r="C25" s="47" t="n">
+      <c r="C25" s="48" t="n">
         <v>0.006855762570378132</v>
       </c>
-      <c r="D25" s="48" t="n">
+      <c r="D25" s="49" t="n">
         <v>0.006855762570378132</v>
       </c>
-      <c r="E25" s="49" t="inlineStr"/>
-      <c r="F25" s="50" t="inlineStr">
+      <c r="E25" s="50" t="inlineStr"/>
+      <c r="F25" s="51" t="inlineStr">
         <is>
           <t>recent</t>
         </is>
       </c>
     </row>
     <row r="26" ht="14" customHeight="1">
-      <c r="A26" s="46" t="inlineStr">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>lag 23</t>
         </is>
       </c>
-      <c r="B26" s="47" t="n">
+      <c r="B26" s="48" t="n">
         <v>0.0111539522300041</v>
       </c>
-      <c r="C26" s="46" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D26" s="51" t="n">
+      <c r="D26" s="52" t="n">
         <v>0.0111539522300041</v>
       </c>
-      <c r="E26" s="49" t="inlineStr"/>
-      <c r="F26" s="50" t="inlineStr">
+      <c r="E26" s="50" t="inlineStr"/>
+      <c r="F26" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
-      <c r="A27" s="46" t="inlineStr">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>lag 24</t>
         </is>
       </c>
-      <c r="B27" s="47" t="n">
+      <c r="B27" s="48" t="n">
         <v>0.01356349181248091</v>
       </c>
-      <c r="C27" s="46" t="inlineStr">
+      <c r="C27" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D27" s="51" t="n">
+      <c r="D27" s="52" t="n">
         <v>0.01356349181248091</v>
       </c>
-      <c r="E27" s="49" t="inlineStr"/>
-      <c r="F27" s="50" t="inlineStr">
+      <c r="E27" s="50" t="inlineStr"/>
+      <c r="F27" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
-      <c r="A28" s="46" t="inlineStr">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>lag 25</t>
         </is>
       </c>
-      <c r="B28" s="47" t="n">
+      <c r="B28" s="48" t="n">
         <v>0.01050675670936246</v>
       </c>
-      <c r="C28" s="46" t="inlineStr">
+      <c r="C28" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D28" s="51" t="n">
+      <c r="D28" s="52" t="n">
         <v>0.01050675670936246</v>
       </c>
-      <c r="E28" s="49" t="inlineStr"/>
-      <c r="F28" s="50" t="inlineStr">
+      <c r="E28" s="50" t="inlineStr"/>
+      <c r="F28" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
-      <c r="A29" s="46" t="inlineStr">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>lag 26</t>
         </is>
       </c>
-      <c r="B29" s="47" t="n">
+      <c r="B29" s="48" t="n">
         <v>0.01034430286365552</v>
       </c>
-      <c r="C29" s="46" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D29" s="51" t="n">
+      <c r="D29" s="52" t="n">
         <v>0.01034430286365552</v>
       </c>
-      <c r="E29" s="49" t="inlineStr"/>
-      <c r="F29" s="50" t="inlineStr">
+      <c r="E29" s="50" t="inlineStr"/>
+      <c r="F29" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
-      <c r="A30" s="46" t="inlineStr">
+      <c r="A30" s="47" t="inlineStr">
         <is>
           <t>lag 27</t>
         </is>
       </c>
-      <c r="B30" s="47" t="n">
+      <c r="B30" s="48" t="n">
         <v>0.008004030604650998</v>
       </c>
-      <c r="C30" s="46" t="inlineStr">
+      <c r="C30" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D30" s="51" t="n">
+      <c r="D30" s="52" t="n">
         <v>0.008004030604650998</v>
       </c>
-      <c r="E30" s="49" t="inlineStr"/>
-      <c r="F30" s="50" t="inlineStr">
+      <c r="E30" s="50" t="inlineStr"/>
+      <c r="F30" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
-      <c r="A31" s="46" t="inlineStr">
+      <c r="A31" s="47" t="inlineStr">
         <is>
           <t>lag 28</t>
         </is>
       </c>
-      <c r="B31" s="47" t="n">
+      <c r="B31" s="48" t="n">
         <v>0.008589939238408145</v>
       </c>
-      <c r="C31" s="46" t="inlineStr">
+      <c r="C31" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D31" s="51" t="n">
+      <c r="D31" s="52" t="n">
         <v>0.008589939238408145</v>
       </c>
-      <c r="E31" s="49" t="inlineStr"/>
-      <c r="F31" s="50" t="inlineStr">
+      <c r="E31" s="50" t="inlineStr"/>
+      <c r="F31" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="32" ht="14" customHeight="1">
-      <c r="A32" s="46" t="inlineStr">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>lag 29</t>
         </is>
       </c>
-      <c r="B32" s="47" t="n">
+      <c r="B32" s="48" t="n">
         <v>0.00795872626437487</v>
       </c>
-      <c r="C32" s="46" t="inlineStr">
+      <c r="C32" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D32" s="51" t="n">
+      <c r="D32" s="52" t="n">
         <v>0.00795872626437487</v>
       </c>
-      <c r="E32" s="49" t="inlineStr"/>
-      <c r="F32" s="50" t="inlineStr">
+      <c r="E32" s="50" t="inlineStr"/>
+      <c r="F32" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="33" ht="14" customHeight="1">
-      <c r="A33" s="46" t="inlineStr">
+      <c r="A33" s="47" t="inlineStr">
         <is>
           <t>lag 30</t>
         </is>
       </c>
-      <c r="B33" s="47" t="n">
+      <c r="B33" s="48" t="n">
         <v>0.006683547200914103</v>
       </c>
-      <c r="C33" s="46" t="inlineStr">
+      <c r="C33" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D33" s="51" t="n">
+      <c r="D33" s="52" t="n">
         <v>0.006683547200914103</v>
       </c>
-      <c r="E33" s="49" t="inlineStr"/>
-      <c r="F33" s="50" t="inlineStr">
+      <c r="E33" s="50" t="inlineStr"/>
+      <c r="F33" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
-      <c r="A34" s="46" t="inlineStr">
+      <c r="A34" s="47" t="inlineStr">
         <is>
           <t>lag 31</t>
         </is>
       </c>
-      <c r="B34" s="47" t="n">
+      <c r="B34" s="48" t="n">
         <v>0.005250505593285775</v>
       </c>
-      <c r="C34" s="46" t="inlineStr">
+      <c r="C34" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D34" s="51" t="n">
+      <c r="D34" s="52" t="n">
         <v>0.005250505593285775</v>
       </c>
-      <c r="E34" s="49" t="inlineStr"/>
-      <c r="F34" s="50" t="inlineStr">
+      <c r="E34" s="50" t="inlineStr"/>
+      <c r="F34" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
-      <c r="A35" s="46" t="inlineStr">
+      <c r="A35" s="47" t="inlineStr">
         <is>
           <t>lag 32</t>
         </is>
       </c>
-      <c r="B35" s="47" t="n">
+      <c r="B35" s="48" t="n">
         <v>0.00568597289102907</v>
       </c>
-      <c r="C35" s="46" t="inlineStr">
+      <c r="C35" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D35" s="51" t="n">
+      <c r="D35" s="52" t="n">
         <v>0.00568597289102907</v>
       </c>
-      <c r="E35" s="49" t="inlineStr"/>
-      <c r="F35" s="50" t="inlineStr">
+      <c r="E35" s="50" t="inlineStr"/>
+      <c r="F35" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
-      <c r="A36" s="46" t="inlineStr">
+      <c r="A36" s="47" t="inlineStr">
         <is>
           <t>lag 33</t>
         </is>
       </c>
-      <c r="B36" s="47" t="n">
+      <c r="B36" s="48" t="n">
         <v>0.00221483942414175</v>
       </c>
-      <c r="C36" s="46" t="inlineStr">
+      <c r="C36" s="47" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="D36" s="51" t="n">
+      <c r="D36" s="52" t="n">
         <v>0.00221483942414175</v>
       </c>
-      <c r="E36" s="49" t="inlineStr"/>
-      <c r="F36" s="50" t="inlineStr">
+      <c r="E36" s="50" t="inlineStr"/>
+      <c r="F36" s="51" t="inlineStr">
         <is>
           <t>full</t>
         </is>
@@ -19288,6 +19921,11 @@
           <t>Col E (Override): if filled, model uses it instead of auto value. Recent curve is preferred for lags 1-16; full curve covers longer lags from 2023 cohorts.</t>
         </is>
       </c>
+      <c r="B38" s="58" t="n"/>
+      <c r="C38" s="58" t="n"/>
+      <c r="D38" s="58" t="n"/>
+      <c r="E38" s="58" t="n"/>
+      <c r="F38" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -19320,6 +19958,9 @@
           <t>Flat Prolongation Rate by Dim  —  EDIT yellow column  (fallback when no payment_no data)</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="58" t="n"/>
+      <c r="D1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -19344,7 +19985,7 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>Base/Private</t>
         </is>
@@ -19352,17 +19993,17 @@
       <c r="B3" s="18" t="n">
         <v>0.458</v>
       </c>
-      <c r="C3" s="52" t="n">
+      <c r="C3" s="53" t="n">
         <v>0.458</v>
       </c>
-      <c r="D3" s="53" t="inlineStr">
+      <c r="D3" s="54" t="inlineStr">
         <is>
           <t>data pool=1655 sec=758</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Base/Premium</t>
         </is>
@@ -19370,17 +20011,17 @@
       <c r="B4" s="18" t="n">
         <v>0.3654</v>
       </c>
-      <c r="C4" s="52" t="n">
+      <c r="C4" s="53" t="n">
         <v>0.3654</v>
       </c>
-      <c r="D4" s="53" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>data pool=1853 sec=677</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>Base/Group</t>
         </is>
@@ -19388,17 +20029,17 @@
       <c r="B5" s="18" t="n">
         <v>0.4462</v>
       </c>
-      <c r="C5" s="52" t="n">
+      <c r="C5" s="53" t="n">
         <v>0.4462</v>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D5" s="54" t="inlineStr">
         <is>
           <t>data pool=7645 sec=3411</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="54" t="inlineStr">
+      <c r="A6" s="55" t="inlineStr">
         <is>
           <t>MT/Private</t>
         </is>
@@ -19406,17 +20047,17 @@
       <c r="B6" s="18" t="n">
         <v>0.6591</v>
       </c>
-      <c r="C6" s="52" t="n">
+      <c r="C6" s="53" t="n">
         <v>0.6591</v>
       </c>
-      <c r="D6" s="53" t="inlineStr">
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>data pool=88 sec=58</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>MT/Premium</t>
         </is>
@@ -19424,10 +20065,10 @@
       <c r="B7" s="18" t="n">
         <v>0.435</v>
       </c>
-      <c r="C7" s="52" t="n">
+      <c r="C7" s="53" t="n">
         <v>0.435</v>
       </c>
-      <c r="D7" s="53" t="inlineStr">
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>hardcoded default (pool=3&lt;15)</t>
         </is>
@@ -19442,10 +20083,10 @@
       <c r="B8" s="18" t="n">
         <v>0.435</v>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="53" t="n">
         <v>0.435</v>
       </c>
-      <c r="D8" s="53" t="inlineStr">
+      <c r="D8" s="54" t="inlineStr">
         <is>
           <t>hardcoded default (pool=7&lt;15)</t>
         </is>
@@ -19457,6 +20098,9 @@
           <t>Global fallback rate (when pool &lt; 15): 0.4345  (pool=11376, sec=4943)</t>
         </is>
       </c>
+      <c r="B9" s="58" t="n"/>
+      <c r="C9" s="58" t="n"/>
+      <c r="D9" s="59" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
@@ -19464,6 +20108,9 @@
           <t>This flat rate is used as a fallback in mode=ext (Jun-Dec 2026) for pool_display calculation. For mode=data/blend the model uses retention_by_renewal[pno] instead.</t>
         </is>
       </c>
+      <c r="B11" s="58" t="n"/>
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -19495,6 +20142,8 @@
           <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
         </is>
       </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -19514,11 +20163,13 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="55" t="inlineStr">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
         </is>
       </c>
+      <c r="B3" s="58" t="n"/>
+      <c r="C3" s="59" t="n"/>
     </row>
     <row r="4" ht="47" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -19606,11 +20257,13 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="55" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>── КОРРЕКЦИЯ AOV ──</t>
         </is>
       </c>
+      <c r="B9" s="58" t="n"/>
+      <c r="C9" s="59" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -19633,11 +20286,13 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="55" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>── РОСТ ЦЕН ──</t>
         </is>
       </c>
+      <c r="B11" s="58" t="n"/>
+      <c r="C11" s="59" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -19685,11 +20340,13 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="55" t="inlineStr">
+      <c r="A15" s="41" t="inlineStr">
         <is>
           <t>── КОРРЕКТИРОВКА RETENTION ──</t>
         </is>
       </c>
+      <c r="B15" s="58" t="n"/>
+      <c r="C15" s="59" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Unified pool+ext model with coverage(k) calibrated from historical data
Architecture: total_sec[T] = pool_sec[T] + (1 - coverage[k]) * ext_full[T]
  - pool_sec = three_pool(pool[T], pool[T+1], pool[T-1]) - actual committed students
  - ext_full = Σ cohort * ext_curve[lag] * EXT_SHARE_SCALE - full cohort estimate
  - coverage[k] = calibrated from 2025 historical data (how full pool[T] is k months ahead)

coverage values: k=1: 99%, k=2: 94%, k=3: 72%, k=4: 56%, k=6: 36%, k=8: 26%, k=12: 5%

Modes:
  data     (Jan-Feb, k=1-2): pool dominates (99-94%)
  data+ext (Mar-Jul, k=3-7): blend (72-31%)
  ext      (Aug-Dec, k=8-12): ext_curve dominates (26-5%)

data_cutoff now defaults to 2025-12-31: train on 2025, predict all 2026

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -190,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -212,55 +212,11 @@
         <color rgb="FFCCCCCC"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -433,8 +389,6 @@
     <xf numFmtId="2" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1039,19 +993,6 @@
           <t>Primary Student Plan Counts (Jan-Dec 2026)  —  EDIT yellow cells</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-      <c r="F1" s="58" t="n"/>
-      <c r="G1" s="58" t="n"/>
-      <c r="H1" s="58" t="n"/>
-      <c r="I1" s="58" t="n"/>
-      <c r="J1" s="58" t="n"/>
-      <c r="K1" s="58" t="n"/>
-      <c r="L1" s="58" t="n"/>
-      <c r="M1" s="58" t="n"/>
-      <c r="N1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
@@ -1453,19 +1394,6 @@
           <t>Edit yellow cells to change the primary student plan, then re-run forecast_2026_v3.py</t>
         </is>
       </c>
-      <c r="B11" s="58" t="n"/>
-      <c r="C11" s="58" t="n"/>
-      <c r="D11" s="58" t="n"/>
-      <c r="E11" s="58" t="n"/>
-      <c r="F11" s="58" t="n"/>
-      <c r="G11" s="58" t="n"/>
-      <c r="H11" s="58" t="n"/>
-      <c r="I11" s="58" t="n"/>
-      <c r="J11" s="58" t="n"/>
-      <c r="K11" s="58" t="n"/>
-      <c r="L11" s="58" t="n"/>
-      <c r="M11" s="58" t="n"/>
-      <c r="N11" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1497,9 +1425,6 @@
           <t>Package Distribution  —  secondary sales Jul-Dec 2025  |  EDIT yellow cells to override</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -7505,9 +7430,6 @@
           <t>Probabilities are auto-normalized per dim in the model. Edit to override distribution.</t>
         </is>
       </c>
-      <c r="B336" s="58" t="n"/>
-      <c r="C336" s="58" t="n"/>
-      <c r="D336" s="59" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="30" t="inlineStr">
@@ -7515,9 +7437,6 @@
           <t>MT dims with thin data use Base/{}-fallback. Base/Group hardcoded fallback: {8: 0.25, 10: 0.14, 32: 0.13, 16: 0.13, 20: 0.09, 4: 0.08, 36: 0.07, 40: 0.06}</t>
         </is>
       </c>
-      <c r="B337" s="58" t="n"/>
-      <c r="C337" s="58" t="n"/>
-      <c r="D337" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7552,11 +7471,6 @@
           <t>Renewal Price per Lesson (base Q3-2025)  —  EDIT yellow cells to override</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-      <c r="F1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -15564,11 +15478,6 @@
           <t>Base period: Q3-2025 (Jul-Sep). Growth factor = (1+3%)^(quarters from Q3-2025). Jan-2026 is Q1-2026 = 2 quarters after Q3-2025, so pgf = 1.0609.</t>
         </is>
       </c>
-      <c r="B336" s="58" t="n"/>
-      <c r="C336" s="58" t="n"/>
-      <c r="D336" s="58" t="n"/>
-      <c r="E336" s="58" t="n"/>
-      <c r="F336" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15604,13 +15513,6 @@
           <t>Retention by (pno, ct, gt, pkg_bucket)  —  Override column takes priority. Fallback: pkg_bucket=ALL (dim-level), then global pno default.</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-      <c r="F1" s="58" t="n"/>
-      <c r="G1" s="58" t="n"/>
-      <c r="H1" s="59" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -15618,13 +15520,6 @@
           <t>Fallback hierarchy: Level1=(pno,ct,gt,pkg) pool&gt;=15  →  Level2=(pno,ct,gt) ALL  →  Level3=global(pno)</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n"/>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="58" t="n"/>
-      <c r="E2" s="58" t="n"/>
-      <c r="F2" s="58" t="n"/>
-      <c r="G2" s="58" t="n"/>
-      <c r="H2" s="59" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -15896,15 +15791,15 @@
         <v>8</v>
       </c>
       <c r="E11" s="36" t="n">
-        <v>0.2083</v>
+        <v>0.2098</v>
       </c>
       <c r="F11" s="18" t="n"/>
       <c r="G11" s="17" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>data pool=144 sec=30</t>
+          <t>data pool=143 sec=30</t>
         </is>
       </c>
     </row>
@@ -16376,15 +16271,15 @@
         <v>8</v>
       </c>
       <c r="E27" s="36" t="n">
-        <v>0.5263</v>
+        <v>0.5357</v>
       </c>
       <c r="F27" s="18" t="n"/>
       <c r="G27" s="21" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>data pool=57 sec=30</t>
+          <t>data pool=56 sec=30</t>
         </is>
       </c>
     </row>
@@ -17066,15 +16961,15 @@
         <v>10</v>
       </c>
       <c r="E50" s="36" t="n">
-        <v>0.6812</v>
+        <v>0.6912</v>
       </c>
       <c r="F50" s="18" t="n"/>
       <c r="G50" s="23" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H50" s="19" t="inlineStr">
         <is>
-          <t>data pool=69 sec=47</t>
+          <t>data pool=68 sec=47</t>
         </is>
       </c>
     </row>
@@ -17968,15 +17863,15 @@
         </is>
       </c>
       <c r="E80" s="18" t="n">
-        <v>0.2903</v>
+        <v>0.2904</v>
       </c>
       <c r="F80" s="18" t="n"/>
       <c r="G80" s="39" t="n">
-        <v>6648</v>
+        <v>6646</v>
       </c>
       <c r="H80" s="19" t="inlineStr">
         <is>
-          <t>data pool=6648 sec=1930  ← Level-2 fallback (ALL pkg)</t>
+          <t>data pool=6646 sec=1930  ← Level-2 fallback (ALL pkg)</t>
         </is>
       </c>
     </row>
@@ -18000,15 +17895,15 @@
         </is>
       </c>
       <c r="E81" s="18" t="n">
-        <v>0.5292</v>
+        <v>0.5294</v>
       </c>
       <c r="F81" s="18" t="n"/>
       <c r="G81" s="39" t="n">
-        <v>2432</v>
+        <v>2431</v>
       </c>
       <c r="H81" s="19" t="inlineStr">
         <is>
-          <t>data pool=2432 sec=1287  ← Level-2 fallback (ALL pkg)</t>
+          <t>data pool=2431 sec=1287  ← Level-2 fallback (ALL pkg)</t>
         </is>
       </c>
     </row>
@@ -18032,15 +17927,15 @@
         </is>
       </c>
       <c r="E82" s="18" t="n">
-        <v>0.6934</v>
+        <v>0.6941000000000001</v>
       </c>
       <c r="F82" s="18" t="n"/>
       <c r="G82" s="39" t="n">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="H82" s="19" t="inlineStr">
         <is>
-          <t>data pool=972 sec=674  ← Level-2 fallback (ALL pkg)</t>
+          <t>data pool=971 sec=674  ← Level-2 fallback (ALL pkg)</t>
         </is>
       </c>
     </row>
@@ -18436,13 +18331,6 @@
           <t>pno=1 = primary (not secondary). pno=2 = first renewal. Override (col F) takes priority over Retention (col E) if non-empty. pkg_bucket rows = Level-1 (pool&gt;=15). ALL rows = Level-2 fallback. For pno&gt;=16 model uses RETENTION_PNO_HIGH=72.0%.</t>
         </is>
       </c>
-      <c r="B96" s="58" t="n"/>
-      <c r="C96" s="58" t="n"/>
-      <c r="D96" s="58" t="n"/>
-      <c r="E96" s="58" t="n"/>
-      <c r="F96" s="58" t="n"/>
-      <c r="G96" s="58" t="n"/>
-      <c r="H96" s="59" t="n"/>
     </row>
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="41" t="inlineStr">
@@ -18450,13 +18338,6 @@
           <t>━━━━━━━━  THREE-POOL RATES  ━━━━━━━━  Hist shares: Present=0.497  Earlier=0.310  Reanim=0.108  —  Edit rates below; scaling applied by forecast_2026_v3.py based on shares sheet</t>
         </is>
       </c>
-      <c r="B98" s="58" t="n"/>
-      <c r="C98" s="58" t="n"/>
-      <c r="D98" s="58" t="n"/>
-      <c r="E98" s="58" t="n"/>
-      <c r="F98" s="58" t="n"/>
-      <c r="G98" s="58" t="n"/>
-      <c r="H98" s="59" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="9" t="inlineStr">
@@ -18515,12 +18396,12 @@
       </c>
       <c r="E100" s="19" t="inlineStr">
         <is>
-          <t>data pool_T=6648 sec=993</t>
+          <t>data pool_T=6646 sec=993</t>
         </is>
       </c>
       <c r="F100" s="19" t="inlineStr">
         <is>
-          <t>data pool_T1=5721 sec=416</t>
+          <t>data pool_T1=5719 sec=416</t>
         </is>
       </c>
       <c r="G100" s="19" t="inlineStr">
@@ -18539,27 +18420,27 @@
         <v>2</v>
       </c>
       <c r="B101" s="18" t="n">
-        <v>0.2636</v>
+        <v>0.2637</v>
       </c>
       <c r="C101" s="18" t="n">
-        <v>0.1394</v>
+        <v>0.1395</v>
       </c>
       <c r="D101" s="18" t="n">
-        <v>0.0546</v>
+        <v>0.0547</v>
       </c>
       <c r="E101" s="19" t="inlineStr">
         <is>
-          <t>data pool_T=2432 sec=641</t>
+          <t>data pool_T=2431 sec=641</t>
         </is>
       </c>
       <c r="F101" s="19" t="inlineStr">
         <is>
-          <t>data pool_T1=2059 sec=287</t>
+          <t>data pool_T1=2058 sec=287</t>
         </is>
       </c>
       <c r="G101" s="19" t="inlineStr">
         <is>
-          <t>data pool_Tm1=2032 sec=111</t>
+          <t>data pool_Tm1=2031 sec=111</t>
         </is>
       </c>
       <c r="H101" s="19" t="inlineStr">
@@ -18573,27 +18454,27 @@
         <v>3</v>
       </c>
       <c r="B102" s="18" t="n">
-        <v>0.3097</v>
+        <v>0.31</v>
       </c>
       <c r="C102" s="18" t="n">
-        <v>0.1633</v>
+        <v>0.1635</v>
       </c>
       <c r="D102" s="18" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="E102" s="19" t="inlineStr">
         <is>
-          <t>data pool_T=972 sec=301</t>
+          <t>data pool_T=971 sec=301</t>
         </is>
       </c>
       <c r="F102" s="19" t="inlineStr">
         <is>
-          <t>data pool_T1=833 sec=136</t>
+          <t>data pool_T1=832 sec=136</t>
         </is>
       </c>
       <c r="G102" s="19" t="inlineStr">
         <is>
-          <t>data pool_Tm1=824 sec=64</t>
+          <t>data pool_Tm1=823 sec=64</t>
         </is>
       </c>
       <c r="H102" s="19" t="inlineStr">
@@ -18948,13 +18829,6 @@
           <t>THREE-POOL section is read by forecast_2026_v3.py for data/blend mode months. rate_present = pool[T]×rate→sec; rate_earlier = pool[T+1]×rate→early-pay; rate_reanim = pool[T-1]×rate→late-pay. Effective rates are scaled by (current_share / hist_share) from the shares sheet.</t>
         </is>
       </c>
-      <c r="B114" s="58" t="n"/>
-      <c r="C114" s="58" t="n"/>
-      <c r="D114" s="58" t="n"/>
-      <c r="E114" s="58" t="n"/>
-      <c r="F114" s="58" t="n"/>
-      <c r="G114" s="58" t="n"/>
-      <c r="H114" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -18988,8 +18862,6 @@
           <t>Segment Shares  —  EDIT yellow column (must sum to 1.0 across all 4 segments)</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -19014,7 +18886,9 @@
           <t>Present</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n"/>
+      <c r="B3" s="18" t="n">
+        <v>0.4971</v>
+      </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid in expected month (paid_M == prev_plan_M)</t>
@@ -19027,7 +18901,9 @@
           <t>Earlier</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n"/>
+      <c r="B4" s="18" t="n">
+        <v>0.3103</v>
+      </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid before expected month (paid_M &lt; prev_plan_M)</t>
@@ -19040,7 +18916,9 @@
           <t>Reanim</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n"/>
+      <c r="B5" s="18" t="n">
+        <v>0.1078</v>
+      </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | Paid after expected month (paid_M &gt; prev_plan_M)</t>
@@ -19053,7 +18931,9 @@
           <t>Upgrades</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n"/>
+      <c r="B6" s="18" t="n">
+        <v>0.0848</v>
+      </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
           <t>data n=4943 | cat_payment = secondary upgrade</t>
@@ -19075,15 +18955,12 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Edit yellow cells. The model normalizes shares automatically if sum != 1.0.</t>
         </is>
       </c>
-      <c r="B9" s="58" t="n"/>
-      <c r="C9" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -19117,11 +18994,6 @@
           <t>Ext-curve (Lag Curve for Future Cohorts)  —  EDIT col E (Override) only if needed</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="58" t="n"/>
-      <c r="E1" s="58" t="n"/>
-      <c r="F1" s="59" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
@@ -19129,11 +19001,6 @@
           <t>Recent (2024-01 to 2025-06): lags 1-22  |  Full fallback (2023-01 to 2025-06): lags 23-33  |  Used by mode=ext (Jun-Dec 2026)</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n"/>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="58" t="n"/>
-      <c r="E2" s="58" t="n"/>
-      <c r="F2" s="59" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
@@ -19174,13 +19041,13 @@
         </is>
       </c>
       <c r="B4" s="48" t="n">
-        <v>0.03243981260767305</v>
+        <v>0.03243713505059474</v>
       </c>
       <c r="C4" s="48" t="n">
-        <v>0.03325380378132611</v>
+        <v>0.03324429452622709</v>
       </c>
       <c r="D4" s="49" t="n">
-        <v>0.03325380378132611</v>
+        <v>0.03324429452622709</v>
       </c>
       <c r="E4" s="50" t="inlineStr"/>
       <c r="F4" s="51" t="inlineStr">
@@ -19196,13 +19063,13 @@
         </is>
       </c>
       <c r="B5" s="48" t="n">
-        <v>0.05565081335823394</v>
+        <v>0.05571452845867907</v>
       </c>
       <c r="C5" s="48" t="n">
-        <v>0.05229594677145271</v>
+        <v>0.05229518891650267</v>
       </c>
       <c r="D5" s="49" t="n">
-        <v>0.05229594677145271</v>
+        <v>0.05229518891650267</v>
       </c>
       <c r="E5" s="50" t="inlineStr"/>
       <c r="F5" s="51" t="inlineStr">
@@ -19218,13 +19085,13 @@
         </is>
       </c>
       <c r="B6" s="48" t="n">
-        <v>0.05740292312901271</v>
+        <v>0.05741896774243076</v>
       </c>
       <c r="C6" s="48" t="n">
-        <v>0.04043051008979147</v>
+        <v>0.04044289435145513</v>
       </c>
       <c r="D6" s="49" t="n">
-        <v>0.04043051008979147</v>
+        <v>0.04044289435145513</v>
       </c>
       <c r="E6" s="50" t="inlineStr"/>
       <c r="F6" s="51" t="inlineStr">
@@ -19240,13 +19107,13 @@
         </is>
       </c>
       <c r="B7" s="48" t="n">
-        <v>0.08721467251692649</v>
+        <v>0.0873644378527494</v>
       </c>
       <c r="C7" s="48" t="n">
-        <v>0.06933519380542201</v>
+        <v>0.06940529352803368</v>
       </c>
       <c r="D7" s="49" t="n">
-        <v>0.06933519380542201</v>
+        <v>0.06940529352803368</v>
       </c>
       <c r="E7" s="50" t="inlineStr"/>
       <c r="F7" s="51" t="inlineStr">
@@ -19262,13 +19129,13 @@
         </is>
       </c>
       <c r="B8" s="48" t="n">
-        <v>0.04908093490622328</v>
+        <v>0.04914905092077902</v>
       </c>
       <c r="C8" s="48" t="n">
-        <v>0.04150558638908253</v>
+        <v>0.04154732608780622</v>
       </c>
       <c r="D8" s="49" t="n">
-        <v>0.04150558638908253</v>
+        <v>0.04154732608780622</v>
       </c>
       <c r="E8" s="50" t="inlineStr"/>
       <c r="F8" s="51" t="inlineStr">
@@ -19284,13 +19151,13 @@
         </is>
       </c>
       <c r="B9" s="48" t="n">
-        <v>0.04107542987799979</v>
+        <v>0.04098805814045773</v>
       </c>
       <c r="C9" s="48" t="n">
-        <v>0.03334841325604449</v>
+        <v>0.03328475403819256</v>
       </c>
       <c r="D9" s="49" t="n">
-        <v>0.03334841325604449</v>
+        <v>0.03328475403819256</v>
       </c>
       <c r="E9" s="50" t="inlineStr"/>
       <c r="F9" s="51" t="inlineStr">
@@ -19306,13 +19173,13 @@
         </is>
       </c>
       <c r="B10" s="48" t="n">
-        <v>0.04132556188857849</v>
+        <v>0.04131669819712211</v>
       </c>
       <c r="C10" s="48" t="n">
-        <v>0.04115337003794277</v>
+        <v>0.04105753983759824</v>
       </c>
       <c r="D10" s="49" t="n">
-        <v>0.04115337003794277</v>
+        <v>0.04105753983759824</v>
       </c>
       <c r="E10" s="50" t="inlineStr"/>
       <c r="F10" s="51" t="inlineStr">
@@ -19328,13 +19195,13 @@
         </is>
       </c>
       <c r="B11" s="48" t="n">
-        <v>0.07794682286006098</v>
+        <v>0.07809455611593051</v>
       </c>
       <c r="C11" s="48" t="n">
-        <v>0.08012093056296371</v>
+        <v>0.08031582560078687</v>
       </c>
       <c r="D11" s="49" t="n">
-        <v>0.08012093056296371</v>
+        <v>0.08031582560078687</v>
       </c>
       <c r="E11" s="50" t="inlineStr"/>
       <c r="F11" s="51" t="inlineStr">
@@ -19350,13 +19217,13 @@
         </is>
       </c>
       <c r="B12" s="48" t="n">
-        <v>0.05219903571086893</v>
+        <v>0.05217172876309011</v>
       </c>
       <c r="C12" s="48" t="n">
-        <v>0.0463728113540315</v>
+        <v>0.04633615413350625</v>
       </c>
       <c r="D12" s="49" t="n">
-        <v>0.0463728113540315</v>
+        <v>0.04633615413350625</v>
       </c>
       <c r="E12" s="50" t="inlineStr"/>
       <c r="F12" s="51" t="inlineStr">
@@ -19372,13 +19239,13 @@
         </is>
       </c>
       <c r="B13" s="48" t="n">
-        <v>0.0263084995491605</v>
+        <v>0.0260696065381613</v>
       </c>
       <c r="C13" s="48" t="n">
-        <v>0.02540345997477899</v>
+        <v>0.02515048563585511</v>
       </c>
       <c r="D13" s="49" t="n">
-        <v>0.02540345997477899</v>
+        <v>0.02515048563585511</v>
       </c>
       <c r="E13" s="50" t="inlineStr"/>
       <c r="F13" s="51" t="inlineStr">
@@ -19394,13 +19261,13 @@
         </is>
       </c>
       <c r="B14" s="48" t="n">
-        <v>0.01694534590044715</v>
+        <v>0.01699454465343098</v>
       </c>
       <c r="C14" s="48" t="n">
-        <v>0.01670792262887267</v>
+        <v>0.01679608349599808</v>
       </c>
       <c r="D14" s="49" t="n">
-        <v>0.01670792262887267</v>
+        <v>0.01679608349599808</v>
       </c>
       <c r="E14" s="50" t="inlineStr"/>
       <c r="F14" s="51" t="inlineStr">
@@ -19416,13 +19283,13 @@
         </is>
       </c>
       <c r="B15" s="48" t="n">
-        <v>0.02311776204827275</v>
+        <v>0.02309468892503899</v>
       </c>
       <c r="C15" s="48" t="n">
-        <v>0.0203014383813916</v>
+        <v>0.02024153317509598</v>
       </c>
       <c r="D15" s="49" t="n">
-        <v>0.0203014383813916</v>
+        <v>0.02024153317509598</v>
       </c>
       <c r="E15" s="50" t="inlineStr"/>
       <c r="F15" s="51" t="inlineStr">
@@ -19438,13 +19305,13 @@
         </is>
       </c>
       <c r="B16" s="48" t="n">
-        <v>0.02009059602064579</v>
+        <v>0.02007651948841538</v>
       </c>
       <c r="C16" s="48" t="n">
-        <v>0.0129558204440133</v>
+        <v>0.01296694907053633</v>
       </c>
       <c r="D16" s="49" t="n">
-        <v>0.0129558204440133</v>
+        <v>0.01296694907053633</v>
       </c>
       <c r="E16" s="50" t="inlineStr"/>
       <c r="F16" s="51" t="inlineStr">
@@ -19460,13 +19327,13 @@
         </is>
       </c>
       <c r="B17" s="48" t="n">
-        <v>0.01442047607706917</v>
+        <v>0.01431560311455341</v>
       </c>
       <c r="C17" s="48" t="n">
-        <v>0.0123686957085169</v>
+        <v>0.01229777847673775</v>
       </c>
       <c r="D17" s="49" t="n">
-        <v>0.0123686957085169</v>
+        <v>0.01229777847673775</v>
       </c>
       <c r="E17" s="50" t="inlineStr"/>
       <c r="F17" s="51" t="inlineStr">
@@ -19482,13 +19349,13 @@
         </is>
       </c>
       <c r="B18" s="48" t="n">
-        <v>0.0190650878142931</v>
+        <v>0.0190703588278369</v>
       </c>
       <c r="C18" s="48" t="n">
-        <v>0.02177364537386275</v>
+        <v>0.02190633303869316</v>
       </c>
       <c r="D18" s="49" t="n">
-        <v>0.02177364537386275</v>
+        <v>0.02190633303869316</v>
       </c>
       <c r="E18" s="50" t="inlineStr"/>
       <c r="F18" s="51" t="inlineStr">
@@ -19504,13 +19371,13 @@
         </is>
       </c>
       <c r="B19" s="48" t="n">
-        <v>0.03493600983148009</v>
+        <v>0.03504565277127267</v>
       </c>
       <c r="C19" s="48" t="n">
-        <v>0.03563806584503205</v>
+        <v>0.03573782562432927</v>
       </c>
       <c r="D19" s="49" t="n">
-        <v>0.03563806584503205</v>
+        <v>0.03573782562432927</v>
       </c>
       <c r="E19" s="50" t="inlineStr"/>
       <c r="F19" s="51" t="inlineStr">
@@ -19526,13 +19393,13 @@
         </is>
       </c>
       <c r="B20" s="48" t="n">
-        <v>0.0265347588824575</v>
+        <v>0.02645519645245165</v>
       </c>
       <c r="C20" s="48" t="n">
-        <v>0.02582494976486335</v>
+        <v>0.02582553763499129</v>
       </c>
       <c r="D20" s="49" t="n">
-        <v>0.02582494976486335</v>
+        <v>0.02582553763499129</v>
       </c>
       <c r="E20" s="50" t="inlineStr"/>
       <c r="F20" s="51" t="inlineStr">
@@ -19548,13 +19415,13 @@
         </is>
       </c>
       <c r="B21" s="48" t="n">
-        <v>0.01720805529257647</v>
+        <v>0.01728150903411541</v>
       </c>
       <c r="C21" s="48" t="n">
-        <v>0.0141590908625448</v>
+        <v>0.01416875856444265</v>
       </c>
       <c r="D21" s="49" t="n">
-        <v>0.0141590908625448</v>
+        <v>0.01416875856444265</v>
       </c>
       <c r="E21" s="50" t="inlineStr"/>
       <c r="F21" s="51" t="inlineStr">
@@ -19570,13 +19437,13 @@
         </is>
       </c>
       <c r="B22" s="48" t="n">
-        <v>0.01112484167561391</v>
+        <v>0.01106552367782303</v>
       </c>
       <c r="C22" s="48" t="n">
-        <v>0.01008889509869752</v>
+        <v>0.009866769426482722</v>
       </c>
       <c r="D22" s="49" t="n">
-        <v>0.01008889509869752</v>
+        <v>0.009866769426482722</v>
       </c>
       <c r="E22" s="50" t="inlineStr"/>
       <c r="F22" s="51" t="inlineStr">
@@ -19592,13 +19459,13 @@
         </is>
       </c>
       <c r="B23" s="48" t="n">
-        <v>0.01020671444500314</v>
+        <v>0.009996584969950595</v>
       </c>
       <c r="C23" s="48" t="n">
-        <v>0.009296585755124544</v>
+        <v>0.008735993396451853</v>
       </c>
       <c r="D23" s="49" t="n">
-        <v>0.009296585755124544</v>
+        <v>0.008735993396451853</v>
       </c>
       <c r="E23" s="50" t="inlineStr"/>
       <c r="F23" s="51" t="inlineStr">
@@ -19614,13 +19481,13 @@
         </is>
       </c>
       <c r="B24" s="48" t="n">
-        <v>0.009025071771145076</v>
+        <v>0.009029106168185884</v>
       </c>
       <c r="C24" s="48" t="n">
-        <v>0.00748335033616986</v>
+        <v>0.007481322848309577</v>
       </c>
       <c r="D24" s="49" t="n">
-        <v>0.00748335033616986</v>
+        <v>0.007481322848309577</v>
       </c>
       <c r="E24" s="50" t="inlineStr"/>
       <c r="F24" s="51" t="inlineStr">
@@ -19636,13 +19503,13 @@
         </is>
       </c>
       <c r="B25" s="48" t="n">
-        <v>0.01282232984589626</v>
+        <v>0.01282446705043657</v>
       </c>
       <c r="C25" s="48" t="n">
-        <v>0.006855762570378132</v>
+        <v>0.006848099433966901</v>
       </c>
       <c r="D25" s="49" t="n">
-        <v>0.006855762570378132</v>
+        <v>0.006848099433966901</v>
       </c>
       <c r="E25" s="50" t="inlineStr"/>
       <c r="F25" s="51" t="inlineStr">
@@ -19658,7 +19525,7 @@
         </is>
       </c>
       <c r="B26" s="48" t="n">
-        <v>0.0111539522300041</v>
+        <v>0.01115738456104733</v>
       </c>
       <c r="C26" s="47" t="inlineStr">
         <is>
@@ -19666,7 +19533,7 @@
         </is>
       </c>
       <c r="D26" s="52" t="n">
-        <v>0.0111539522300041</v>
+        <v>0.01115738456104733</v>
       </c>
       <c r="E26" s="50" t="inlineStr"/>
       <c r="F26" s="51" t="inlineStr">
@@ -19682,7 +19549,7 @@
         </is>
       </c>
       <c r="B27" s="48" t="n">
-        <v>0.01356349181248091</v>
+        <v>0.01367050648243216</v>
       </c>
       <c r="C27" s="47" t="inlineStr">
         <is>
@@ -19690,7 +19557,7 @@
         </is>
       </c>
       <c r="D27" s="52" t="n">
-        <v>0.01356349181248091</v>
+        <v>0.01367050648243216</v>
       </c>
       <c r="E27" s="50" t="inlineStr"/>
       <c r="F27" s="51" t="inlineStr">
@@ -19706,7 +19573,7 @@
         </is>
       </c>
       <c r="B28" s="48" t="n">
-        <v>0.01050675670936246</v>
+        <v>0.01051452201970425</v>
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
@@ -19714,7 +19581,7 @@
         </is>
       </c>
       <c r="D28" s="52" t="n">
-        <v>0.01050675670936246</v>
+        <v>0.01051452201970425</v>
       </c>
       <c r="E28" s="50" t="inlineStr"/>
       <c r="F28" s="51" t="inlineStr">
@@ -19730,7 +19597,7 @@
         </is>
       </c>
       <c r="B29" s="48" t="n">
-        <v>0.01034430286365552</v>
+        <v>0.01035138989421092</v>
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
@@ -19738,7 +19605,7 @@
         </is>
       </c>
       <c r="D29" s="52" t="n">
-        <v>0.01034430286365552</v>
+        <v>0.01035138989421092</v>
       </c>
       <c r="E29" s="50" t="inlineStr"/>
       <c r="F29" s="51" t="inlineStr">
@@ -19754,7 +19621,7 @@
         </is>
       </c>
       <c r="B30" s="48" t="n">
-        <v>0.008004030604650998</v>
+        <v>0.008010068655063081</v>
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
@@ -19762,7 +19629,7 @@
         </is>
       </c>
       <c r="D30" s="52" t="n">
-        <v>0.008004030604650998</v>
+        <v>0.008010068655063081</v>
       </c>
       <c r="E30" s="50" t="inlineStr"/>
       <c r="F30" s="51" t="inlineStr">
@@ -19778,7 +19645,7 @@
         </is>
       </c>
       <c r="B31" s="48" t="n">
-        <v>0.008589939238408145</v>
+        <v>0.008596302308117809</v>
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
@@ -19786,7 +19653,7 @@
         </is>
       </c>
       <c r="D31" s="52" t="n">
-        <v>0.008589939238408145</v>
+        <v>0.008596302308117809</v>
       </c>
       <c r="E31" s="50" t="inlineStr"/>
       <c r="F31" s="51" t="inlineStr">
@@ -19802,7 +19669,7 @@
         </is>
       </c>
       <c r="B32" s="48" t="n">
-        <v>0.00795872626437487</v>
+        <v>0.00795888431053699</v>
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
@@ -19810,7 +19677,7 @@
         </is>
       </c>
       <c r="D32" s="52" t="n">
-        <v>0.00795872626437487</v>
+        <v>0.00795888431053699</v>
       </c>
       <c r="E32" s="50" t="inlineStr"/>
       <c r="F32" s="51" t="inlineStr">
@@ -19826,7 +19693,7 @@
         </is>
       </c>
       <c r="B33" s="48" t="n">
-        <v>0.006683547200914103</v>
+        <v>0.006688722350730599</v>
       </c>
       <c r="C33" s="47" t="inlineStr">
         <is>
@@ -19834,7 +19701,7 @@
         </is>
       </c>
       <c r="D33" s="52" t="n">
-        <v>0.006683547200914103</v>
+        <v>0.006688722350730599</v>
       </c>
       <c r="E33" s="50" t="inlineStr"/>
       <c r="F33" s="51" t="inlineStr">
@@ -19850,7 +19717,7 @@
         </is>
       </c>
       <c r="B34" s="48" t="n">
-        <v>0.005250505593285775</v>
+        <v>0.005252912679748321</v>
       </c>
       <c r="C34" s="47" t="inlineStr">
         <is>
@@ -19858,7 +19725,7 @@
         </is>
       </c>
       <c r="D34" s="52" t="n">
-        <v>0.005250505593285775</v>
+        <v>0.005252912679748321</v>
       </c>
       <c r="E34" s="50" t="inlineStr"/>
       <c r="F34" s="51" t="inlineStr">
@@ -19921,11 +19788,6 @@
           <t>Col E (Override): if filled, model uses it instead of auto value. Recent curve is preferred for lags 1-16; full curve covers longer lags from 2023 cohorts.</t>
         </is>
       </c>
-      <c r="B38" s="58" t="n"/>
-      <c r="C38" s="58" t="n"/>
-      <c r="D38" s="58" t="n"/>
-      <c r="E38" s="58" t="n"/>
-      <c r="F38" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -19958,9 +19820,6 @@
           <t>Flat Prolongation Rate by Dim  —  EDIT yellow column  (fallback when no payment_no data)</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="58" t="n"/>
-      <c r="D1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -19991,14 +19850,14 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>0.458</v>
+        <v>0.4583</v>
       </c>
       <c r="C3" s="53" t="n">
-        <v>0.458</v>
+        <v>0.4583</v>
       </c>
       <c r="D3" s="54" t="inlineStr">
         <is>
-          <t>data pool=1655 sec=758</t>
+          <t>data pool=1654 sec=758</t>
         </is>
       </c>
     </row>
@@ -20009,14 +19868,14 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>0.3654</v>
+        <v>0.3656</v>
       </c>
       <c r="C4" s="53" t="n">
-        <v>0.3654</v>
+        <v>0.3656</v>
       </c>
       <c r="D4" s="54" t="inlineStr">
         <is>
-          <t>data pool=1853 sec=677</t>
+          <t>data pool=1852 sec=677</t>
         </is>
       </c>
     </row>
@@ -20034,7 +19893,7 @@
       </c>
       <c r="D5" s="54" t="inlineStr">
         <is>
-          <t>data pool=7645 sec=3411</t>
+          <t>data pool=7644 sec=3411</t>
         </is>
       </c>
     </row>
@@ -20045,14 +19904,14 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>0.6591</v>
+        <v>0.6667</v>
       </c>
       <c r="C6" s="53" t="n">
-        <v>0.6591</v>
+        <v>0.6667</v>
       </c>
       <c r="D6" s="54" t="inlineStr">
         <is>
-          <t>data pool=88 sec=58</t>
+          <t>data pool=87 sec=58</t>
         </is>
       </c>
     </row>
@@ -20095,12 +19954,9 @@
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Global fallback rate (when pool &lt; 15): 0.4345  (pool=11376, sec=4943)</t>
-        </is>
-      </c>
-      <c r="B9" s="58" t="n"/>
-      <c r="C9" s="58" t="n"/>
-      <c r="D9" s="59" t="n"/>
+          <t>Global fallback rate (when pool &lt; 15): 0.4347  (pool=11372, sec=4943)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
@@ -20108,9 +19964,6 @@
           <t>This flat rate is used as a fallback in mode=ext (Jun-Dec 2026) for pool_display calculation. For mode=data/blend the model uses retention_by_renewal[pno] instead.</t>
         </is>
       </c>
-      <c r="B11" s="58" t="n"/>
-      <c r="C11" s="58" t="n"/>
-      <c r="D11" s="59" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -20142,8 +19995,6 @@
           <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
         </is>
       </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="59" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -20168,8 +20019,6 @@
           <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
         </is>
       </c>
-      <c r="B3" s="58" t="n"/>
-      <c r="C3" s="59" t="n"/>
     </row>
     <row r="4" ht="47" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -20179,7 +20028,7 @@
       </c>
       <c r="B4" s="56" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C4" s="30" t="inlineStr">
@@ -20262,8 +20111,6 @@
           <t>── КОРРЕКЦИЯ AOV ──</t>
         </is>
       </c>
-      <c r="B9" s="58" t="n"/>
-      <c r="C9" s="59" t="n"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -20291,8 +20138,6 @@
           <t>── РОСТ ЦЕН ──</t>
         </is>
       </c>
-      <c r="B11" s="58" t="n"/>
-      <c r="C11" s="59" t="n"/>
     </row>
     <row r="12" ht="21" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -20345,8 +20190,6 @@
           <t>── КОРРЕКТИРОВКА RETENTION ──</t>
         </is>
       </c>
-      <c r="B15" s="58" t="n"/>
-      <c r="C15" s="59" t="n"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add pno-bucket AOV calibration: pool=pno-weighted, ext_hist=Q4avg, ext_plan=pno2
Three-component AOV model:
  pool_sec  -> pno-weighted AOV from pool_by_pno distribution
  ext_hist  -> direct_aov_base Q4-2025 average (historical cohorts, mixed pno)
  ext_plan  -> direct_aov_by_pno[(ct,gt,2)] = pno=2 AOV (plan cohorts, first renewals)

Calibrated AOV by pno bucket (Base/Group):
  pno=2: $161, pno=3-4: $152, pno=5-7: $115, pno=8-12: $82, pno=13+: $63

Key insight: AOV decreases with pno (loyal students buy smaller maintenance packages).
First renewals (pno=2) have highest AOV - new students commit with large packages.
Pool for Jan-Feb is mostly pno=2-4 -> pno-weighted AOV > flat Q4 average.

New Excel sheet: aov_by_pno (Dim | pno_bucket | Calibrated | Override | n_samples)
Saves PRE_FINAL backup locally.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ext_curve" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rates" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aov_by_pno" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -216,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -387,6 +389,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -962,6 +985,838 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>AOV by Dim × pno_bucket  —  Q4-2025 calibration  |  EDIT yellow Override column (col D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>pno=2 = first renewal; 3-4 = 2nd-3rd; 5-7 = 4th-6th; 8-12 = 7th-11th; 13+ = veteran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Dim</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>pno_bucket</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>AOV (calibrated)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>n_samples</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Note / Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="n">
+        <v>316</v>
+      </c>
+      <c r="D4" s="60" t="n"/>
+      <c r="E4" s="17" t="n">
+        <v>140</v>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=140</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C5" s="59" t="n">
+        <v>312.24</v>
+      </c>
+      <c r="D5" s="60" t="n"/>
+      <c r="E5" s="17" t="n">
+        <v>151</v>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=151</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B6" s="58" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C6" s="59" t="n">
+        <v>233.04</v>
+      </c>
+      <c r="D6" s="60" t="n"/>
+      <c r="E6" s="17" t="n">
+        <v>63</v>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=63</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C7" s="59" t="n">
+        <v>165</v>
+      </c>
+      <c r="D7" s="60" t="n"/>
+      <c r="E7" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C8" s="59" t="n">
+        <v>287.79</v>
+      </c>
+      <c r="D8" s="60" t="n"/>
+      <c r="E8" s="58" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=6&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C9" s="59" t="n">
+        <v>201.91</v>
+      </c>
+      <c r="D9" s="60" t="n"/>
+      <c r="E9" s="21" t="n">
+        <v>290</v>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=290</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C10" s="59" t="n">
+        <v>162.32</v>
+      </c>
+      <c r="D10" s="60" t="n"/>
+      <c r="E10" s="21" t="n">
+        <v>135</v>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=135</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C11" s="59" t="n">
+        <v>131.88</v>
+      </c>
+      <c r="D11" s="60" t="n"/>
+      <c r="E11" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C12" s="59" t="n">
+        <v>187</v>
+      </c>
+      <c r="D12" s="60" t="n"/>
+      <c r="E12" s="61" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C13" s="59" t="n">
+        <v>187</v>
+      </c>
+      <c r="D13" s="60" t="n"/>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B14" s="62" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C14" s="59" t="n">
+        <v>168.54</v>
+      </c>
+      <c r="D14" s="60" t="n"/>
+      <c r="E14" s="23" t="n">
+        <v>553</v>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=553</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B15" s="62" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C15" s="59" t="n">
+        <v>161.87</v>
+      </c>
+      <c r="D15" s="60" t="n"/>
+      <c r="E15" s="23" t="n">
+        <v>712</v>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=712</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B16" s="62" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C16" s="59" t="n">
+        <v>117.55</v>
+      </c>
+      <c r="D16" s="60" t="n"/>
+      <c r="E16" s="23" t="n">
+        <v>290</v>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=290</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C17" s="59" t="n">
+        <v>84.62</v>
+      </c>
+      <c r="D17" s="60" t="n"/>
+      <c r="E17" s="23" t="n">
+        <v>106</v>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=106</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B18" s="62" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C18" s="59" t="n">
+        <v>78.53</v>
+      </c>
+      <c r="D18" s="60" t="n"/>
+      <c r="E18" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=22</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B19" s="63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C19" s="59" t="n">
+        <v>285.07</v>
+      </c>
+      <c r="D19" s="60" t="n"/>
+      <c r="E19" s="25" t="n">
+        <v>41</v>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=41</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="n">
+        <v>250.99</v>
+      </c>
+      <c r="D20" s="60" t="n"/>
+      <c r="E20" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>Q4-2025 data n=12</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C21" s="59" t="n">
+        <v>271.51</v>
+      </c>
+      <c r="D21" s="60" t="n"/>
+      <c r="E21" s="63" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=2&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B22" s="63" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="n">
+        <v>271.51</v>
+      </c>
+      <c r="D22" s="60" t="n"/>
+      <c r="E22" s="63" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="n">
+        <v>271.51</v>
+      </c>
+      <c r="D23" s="60" t="n"/>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B24" s="64" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D24" s="60" t="n"/>
+      <c r="E24" s="64" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=1&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B25" s="64" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D25" s="60" t="n"/>
+      <c r="E25" s="64" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=2&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B26" s="64" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C26" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D26" s="60" t="n"/>
+      <c r="E26" s="64" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B27" s="64" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C27" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D27" s="60" t="n"/>
+      <c r="E27" s="64" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B28" s="64" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C28" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D28" s="60" t="n"/>
+      <c r="E28" s="64" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B29" s="47" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C29" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D29" s="60" t="n"/>
+      <c r="E29" s="47" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=1&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B30" s="47" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="C30" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D30" s="60" t="n"/>
+      <c r="E30" s="47" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=3&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="C31" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D31" s="60" t="n"/>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F31" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B32" s="47" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="C32" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D32" s="60" t="n"/>
+      <c r="E32" s="47" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="inlineStr">
+        <is>
+          <t>13+</t>
+        </is>
+      </c>
+      <c r="C33" s="59" t="n">
+        <v>180.45</v>
+      </c>
+      <c r="D33" s="60" t="n"/>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="F33" s="19" t="inlineStr">
+        <is>
+          <t>dim fallback n=0&lt;10</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>Col C = calibrated from Q4-2025 data (or dim fallback if n&lt;10). Col D = Override: if filled, forecast_2026_v3.py uses it instead. MT dims with thin data fall back to dim average.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A35:F35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fix PLAN_COHORT_START + update June 2026 plan to negative scenario
Bug fix: PLAN_COHORT_START now = data_cutoff month (2026-06) instead of
cutoff+1 (2026-07). Current month is partial in CSV — primary sales must
come from plan_counts, not CSV data.

June 2026 plan_counts updated: 396 → 2007 (from negative scenario shares).
This correctly propagates June cohort into Jul-Dec 2026 secondary forecast.

Impact: TOTAL 2026 updated to $2,433,071 / 11,690 sales
(was $2,312,062 / 11,185 with old June=396)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/forecast_inputs_2026.xlsx
+++ b/forecast_inputs_2026.xlsx
@@ -8,14 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plan_counts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="package_dist" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="renewal_price" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="retention_by_renewal" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="shares" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ext_curve" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rates" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plan_counts_negative" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="plan_counts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="package_dist" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="renewal_price" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="retention_by_renewal" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="shares" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ext_curve" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rates" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +25,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="$#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.000%"/>
+    <numFmt numFmtId="168" formatCode="+#,##0;-#,##0;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -120,6 +122,48 @@
       <b val="1"/>
       <color rgb="FF212529"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF1B2A4A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="FF1B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <color rgb="FF1B2A4A"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="14">
@@ -260,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -435,6 +479,72 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="20" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="19" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="19" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1008,7 +1118,1253 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
+        </is>
+      </c>
+      <c r="B1" s="58" t="n"/>
+      <c r="C1" s="59" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Параметр</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Описание / Как влияет</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
+        </is>
+      </c>
+      <c r="B3" s="58" t="n"/>
+      <c r="C3" s="59" t="n"/>
+    </row>
+    <row r="4" ht="47" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>data_cutoff</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Дата последних данных. Месяцы ДО этой даты используют режим data/blend. Например: 2024-12-31 = данные по декабрь 2024, прогноз с января 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>cal_window_start</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Начало окна калибровки рейтов/долей/AOV. Формат: YYYY-MM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>cal_window_end</t>
+        </is>
+      </c>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>Конец окна калибровки. По умолчанию — последний полный месяц до data_cutoff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>forecast_start</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Первый месяц прогноза. Формат: YYYY-MM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="29" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>forecast_end</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Последний месяц прогноза. Например: 2027-05 = прогноз на 12 мес. вперёд от data_cutoff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>── КОРРЕКЦИЯ AOV ──</t>
+        </is>
+      </c>
+      <c r="B9" s="58" t="n"/>
+      <c r="C9" s="59" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>aov_adjustment_factor</t>
+        </is>
+      </c>
+      <c r="B10" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>❗ ПОЧЕМУ AOV может отличаться от факта:
+1. Цены calibrated на среднем (mean) — чувствительно к выбросам и сезонности.
+2. Пакеты pkg=999 (кастомные) исключены из калибровки — реальный AOV выше.
+3. Распределение пакетов июл-дек 2025 может отличаться от 2026.
+→ Коэффициент 1.10 = скорректировать выручку на 10% (бэктест: Jan 2026 = -0.2%).
+→ Поставь 1.0 чтобы без коррекции. Меняй под обновлённые данные.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>── РОСТ ЦЕН ──</t>
+        </is>
+      </c>
+      <c r="B11" s="58" t="n"/>
+      <c r="C11" s="59" t="n"/>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>price_growth_pct_per_quarter</t>
+        </is>
+      </c>
+      <c r="B12" s="57" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Рост цены за урок в квартал (3% = +3%/квартал). База = Q3 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>price_base_year</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Год базового периода для роста цен.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="43" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>price_base_quarter</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Квартал базового периода (4 = Q4 = окт-дек, рекомендуется). Диагностика: Q3→Q4 рост +15%, поэтому Q4 = более точная база для 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>── КОРРЕКТИРОВКА RETENTION ──</t>
+        </is>
+      </c>
+      <c r="B15" s="58" t="n"/>
+      <c r="C15" s="59" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>retention_adjustment</t>
+        </is>
+      </c>
+      <c r="B16" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>❗ ТРЕНД СНИЖЕНИЯ RETENTION:
+May 2026 actual: retention=38.4% vs калибровка Jul-Dec 2025: 43.6% (-12%).
+Retention постепенно снижается год к году.
+→ 0.88 = умножить все retention[pno] на 0.88 (-12%)
+→ 1.0  = без коррекции (использовать 2025 ставки)
+Рекомендация для 2026 прогноза: попробуй 0.88-0.92.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>plan_counts_negative  —  Primary student plan (scenario: new inputs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>SOURCE DATA (from planning inputs — for verification)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="62" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="62" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="D3" s="62" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="E3" s="62" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="F3" s="62" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="G3" s="62" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="H3" s="62" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="I3" s="62" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="J3" s="62" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="K3" s="62" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="L3" s="62" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="M3" s="62" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="N3" s="62" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t>Total primary plan</t>
+        </is>
+      </c>
+      <c r="B4" s="64" t="n">
+        <v>1573</v>
+      </c>
+      <c r="C4" s="64" t="n">
+        <v>1127</v>
+      </c>
+      <c r="D4" s="64" t="n">
+        <v>816</v>
+      </c>
+      <c r="E4" s="64" t="n">
+        <v>1318</v>
+      </c>
+      <c r="F4" s="64" t="n">
+        <v>1557</v>
+      </c>
+      <c r="G4" s="64" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H4" s="64" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I4" s="64" t="n">
+        <v>1467</v>
+      </c>
+      <c r="J4" s="64" t="n">
+        <v>1354</v>
+      </c>
+      <c r="K4" s="64" t="n">
+        <v>1284</v>
+      </c>
+      <c r="L4" s="64" t="n">
+        <v>1420</v>
+      </c>
+      <c r="M4" s="64" t="n">
+        <v>1450</v>
+      </c>
+      <c r="N4" s="64" t="n">
+        <v>17223</v>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="65" t="inlineStr">
+        <is>
+          <t>Share Primary Base %</t>
+        </is>
+      </c>
+      <c r="B5" s="66" t="n">
+        <v>0.8109999999999999</v>
+      </c>
+      <c r="C5" s="66" t="n">
+        <v>0.584</v>
+      </c>
+      <c r="D5" s="66" t="n">
+        <v>0.5760000000000001</v>
+      </c>
+      <c r="E5" s="66" t="n">
+        <v>0.6142</v>
+      </c>
+      <c r="F5" s="66" t="n">
+        <v>0.5760000000000001</v>
+      </c>
+      <c r="G5" s="66" t="n">
+        <v>0.5760000000000001</v>
+      </c>
+      <c r="H5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="I5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="J5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="K5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="L5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="M5" s="66" t="n">
+        <v>0.472</v>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>Share Primary MT %</t>
+        </is>
+      </c>
+      <c r="B6" s="68" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="C6" s="68" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="D6" s="68" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="E6" s="68" t="n">
+        <v>0.3858</v>
+      </c>
+      <c r="F6" s="68" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="G6" s="68" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="H6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="I6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="J6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="K6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="L6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="M6" s="68" t="n">
+        <v>0.528</v>
+      </c>
+    </row>
+    <row r="7" ht="13" customHeight="1">
+      <c r="A7" s="69" t="inlineStr">
+        <is>
+          <t>Sharing ind BF</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="C7" s="70" t="n">
+        <v>0.208</v>
+      </c>
+      <c r="D7" s="70" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="E7" s="70" t="n">
+        <v>0.3728</v>
+      </c>
+      <c r="F7" s="70" t="n">
+        <v>0.4054</v>
+      </c>
+      <c r="G7" s="70" t="n">
+        <v>0.3202</v>
+      </c>
+      <c r="H7" s="70" t="n">
+        <v>0.3251</v>
+      </c>
+      <c r="I7" s="70" t="n">
+        <v>0.3512</v>
+      </c>
+      <c r="J7" s="70" t="n">
+        <v>0.3271</v>
+      </c>
+      <c r="K7" s="70" t="n">
+        <v>0.3021</v>
+      </c>
+      <c r="L7" s="70" t="n">
+        <v>0.3264</v>
+      </c>
+      <c r="M7" s="70" t="n">
+        <v>0.3215</v>
+      </c>
+    </row>
+    <row r="8" ht="13" customHeight="1">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>Sharing mini BF</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="C8" s="70" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="D8" s="70" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="E8" s="70" t="n">
+        <v>0.2687</v>
+      </c>
+      <c r="F8" s="70" t="n">
+        <v>0.2716</v>
+      </c>
+      <c r="G8" s="70" t="n">
+        <v>0.3595</v>
+      </c>
+      <c r="H8" s="70" t="n">
+        <v>0.3532</v>
+      </c>
+      <c r="I8" s="70" t="n">
+        <v>0.3347</v>
+      </c>
+      <c r="J8" s="70" t="n">
+        <v>0.3531</v>
+      </c>
+      <c r="K8" s="70" t="n">
+        <v>0.3618</v>
+      </c>
+      <c r="L8" s="70" t="n">
+        <v>0.3685</v>
+      </c>
+      <c r="M8" s="70" t="n">
+        <v>0.3782</v>
+      </c>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="69" t="inlineStr">
+        <is>
+          <t>Sharing group BF</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="C9" s="70" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="D9" s="70" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="E9" s="70" t="n">
+        <v>0.3585</v>
+      </c>
+      <c r="F9" s="70" t="n">
+        <v>0.323</v>
+      </c>
+      <c r="G9" s="70" t="n">
+        <v>0.3203</v>
+      </c>
+      <c r="H9" s="70" t="n">
+        <v>0.3217</v>
+      </c>
+      <c r="I9" s="70" t="n">
+        <v>0.314</v>
+      </c>
+      <c r="J9" s="70" t="n">
+        <v>0.3198</v>
+      </c>
+      <c r="K9" s="70" t="n">
+        <v>0.3361</v>
+      </c>
+      <c r="L9" s="70" t="n">
+        <v>0.3051</v>
+      </c>
+      <c r="M9" s="70" t="n">
+        <v>0.3002</v>
+      </c>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>Sharing ind MT</t>
+        </is>
+      </c>
+      <c r="B10" s="72" t="n">
+        <v>0.4245</v>
+      </c>
+      <c r="C10" s="72" t="n">
+        <v>0.5357999999999999</v>
+      </c>
+      <c r="D10" s="72" t="n">
+        <v>0.4019</v>
+      </c>
+      <c r="E10" s="72" t="n">
+        <v>0.3736</v>
+      </c>
+      <c r="F10" s="72" t="n">
+        <v>0.4363</v>
+      </c>
+      <c r="G10" s="72" t="n">
+        <v>0.3648</v>
+      </c>
+      <c r="H10" s="72" t="n">
+        <v>0.3171</v>
+      </c>
+      <c r="I10" s="72" t="n">
+        <v>0.3305</v>
+      </c>
+      <c r="J10" s="72" t="n">
+        <v>0.3227</v>
+      </c>
+      <c r="K10" s="72" t="n">
+        <v>0.3337</v>
+      </c>
+      <c r="L10" s="72" t="n">
+        <v>0.324</v>
+      </c>
+      <c r="M10" s="72" t="n">
+        <v>0.3157</v>
+      </c>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="71" t="inlineStr">
+        <is>
+          <t>Sharing mini MT</t>
+        </is>
+      </c>
+      <c r="B11" s="72" t="n">
+        <v>0.2764</v>
+      </c>
+      <c r="C11" s="72" t="n">
+        <v>0.2499</v>
+      </c>
+      <c r="D11" s="72" t="n">
+        <v>0.3573</v>
+      </c>
+      <c r="E11" s="72" t="n">
+        <v>0.344</v>
+      </c>
+      <c r="F11" s="72" t="n">
+        <v>0.3397</v>
+      </c>
+      <c r="G11" s="72" t="n">
+        <v>0.4005</v>
+      </c>
+      <c r="H11" s="72" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="I11" s="72" t="n">
+        <v>0.4043</v>
+      </c>
+      <c r="J11" s="72" t="n">
+        <v>0.4004</v>
+      </c>
+      <c r="K11" s="72" t="n">
+        <v>0.3947</v>
+      </c>
+      <c r="L11" s="72" t="n">
+        <v>0.4005</v>
+      </c>
+      <c r="M11" s="72" t="n">
+        <v>0.3976</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="71" t="inlineStr">
+        <is>
+          <t>Sharing group MT</t>
+        </is>
+      </c>
+      <c r="B12" s="72" t="n">
+        <v>0.2991</v>
+      </c>
+      <c r="C12" s="72" t="n">
+        <v>0.2143</v>
+      </c>
+      <c r="D12" s="72" t="n">
+        <v>0.2408</v>
+      </c>
+      <c r="E12" s="72" t="n">
+        <v>0.2824</v>
+      </c>
+      <c r="F12" s="72" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="G12" s="72" t="n">
+        <v>0.2347</v>
+      </c>
+      <c r="H12" s="72" t="n">
+        <v>0.2543</v>
+      </c>
+      <c r="I12" s="72" t="n">
+        <v>0.2652</v>
+      </c>
+      <c r="J12" s="72" t="n">
+        <v>0.2769</v>
+      </c>
+      <c r="K12" s="72" t="n">
+        <v>0.2717</v>
+      </c>
+      <c r="L12" s="72" t="n">
+        <v>0.2755</v>
+      </c>
+      <c r="M12" s="72" t="n">
+        <v>0.2866</v>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="61" t="inlineStr">
+        <is>
+          <t>COMPUTED PLAN BY DIM  (ready to paste into plan_counts sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="62" t="inlineStr">
+        <is>
+          <t>Dim \ Month</t>
+        </is>
+      </c>
+      <c r="B15" s="62" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C15" s="62" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D15" s="62" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="E15" s="62" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="F15" s="62" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="H15" s="62" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="I15" s="62" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="J15" s="62" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="K15" s="62" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L15" s="62" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M15" s="62" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="N15" s="62" t="inlineStr">
+        <is>
+          <t>Year Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="73" t="inlineStr">
+        <is>
+          <t>Base/Private</t>
+        </is>
+      </c>
+      <c r="B16" s="74" t="n">
+        <v>216</v>
+      </c>
+      <c r="C16" s="74" t="n">
+        <v>139</v>
+      </c>
+      <c r="D16" s="74" t="n">
+        <v>73</v>
+      </c>
+      <c r="E16" s="74" t="n">
+        <v>302</v>
+      </c>
+      <c r="F16" s="74" t="n">
+        <v>364</v>
+      </c>
+      <c r="G16" s="74" t="n">
+        <v>370</v>
+      </c>
+      <c r="H16" s="74" t="n">
+        <v>284</v>
+      </c>
+      <c r="I16" s="74" t="n">
+        <v>243</v>
+      </c>
+      <c r="J16" s="74" t="n">
+        <v>209</v>
+      </c>
+      <c r="K16" s="74" t="n">
+        <v>183</v>
+      </c>
+      <c r="L16" s="74" t="n">
+        <v>219</v>
+      </c>
+      <c r="M16" s="74" t="n">
+        <v>220</v>
+      </c>
+      <c r="N16" s="75" t="n">
+        <v>2822</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="73" t="inlineStr">
+        <is>
+          <t>Base/Premium</t>
+        </is>
+      </c>
+      <c r="B17" s="74" t="n">
+        <v>456</v>
+      </c>
+      <c r="C17" s="74" t="n">
+        <v>206</v>
+      </c>
+      <c r="D17" s="74" t="n">
+        <v>170</v>
+      </c>
+      <c r="E17" s="74" t="n">
+        <v>218</v>
+      </c>
+      <c r="F17" s="74" t="n">
+        <v>244</v>
+      </c>
+      <c r="G17" s="74" t="n">
+        <v>416</v>
+      </c>
+      <c r="H17" s="74" t="n">
+        <v>308</v>
+      </c>
+      <c r="I17" s="74" t="n">
+        <v>232</v>
+      </c>
+      <c r="J17" s="74" t="n">
+        <v>226</v>
+      </c>
+      <c r="K17" s="74" t="n">
+        <v>219</v>
+      </c>
+      <c r="L17" s="74" t="n">
+        <v>247</v>
+      </c>
+      <c r="M17" s="74" t="n">
+        <v>259</v>
+      </c>
+      <c r="N17" s="75" t="n">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="73" t="inlineStr">
+        <is>
+          <t>Base/Group</t>
+        </is>
+      </c>
+      <c r="B18" s="74" t="n">
+        <v>604</v>
+      </c>
+      <c r="C18" s="74" t="n">
+        <v>313</v>
+      </c>
+      <c r="D18" s="74" t="n">
+        <v>227</v>
+      </c>
+      <c r="E18" s="74" t="n">
+        <v>290</v>
+      </c>
+      <c r="F18" s="74" t="n">
+        <v>290</v>
+      </c>
+      <c r="G18" s="74" t="n">
+        <v>370</v>
+      </c>
+      <c r="H18" s="74" t="n">
+        <v>281</v>
+      </c>
+      <c r="I18" s="74" t="n">
+        <v>217</v>
+      </c>
+      <c r="J18" s="74" t="n">
+        <v>204</v>
+      </c>
+      <c r="K18" s="74" t="n">
+        <v>204</v>
+      </c>
+      <c r="L18" s="74" t="n">
+        <v>204</v>
+      </c>
+      <c r="M18" s="74" t="n">
+        <v>205</v>
+      </c>
+      <c r="N18" s="75" t="n">
+        <v>3409</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="76" t="inlineStr">
+        <is>
+          <t>MT/Private</t>
+        </is>
+      </c>
+      <c r="B19" s="77" t="n">
+        <v>126</v>
+      </c>
+      <c r="C19" s="77" t="n">
+        <v>251</v>
+      </c>
+      <c r="D19" s="77" t="n">
+        <v>139</v>
+      </c>
+      <c r="E19" s="77" t="n">
+        <v>190</v>
+      </c>
+      <c r="F19" s="77" t="n">
+        <v>288</v>
+      </c>
+      <c r="G19" s="77" t="n">
+        <v>310</v>
+      </c>
+      <c r="H19" s="77" t="n">
+        <v>310</v>
+      </c>
+      <c r="I19" s="77" t="n">
+        <v>256</v>
+      </c>
+      <c r="J19" s="77" t="n">
+        <v>231</v>
+      </c>
+      <c r="K19" s="77" t="n">
+        <v>226</v>
+      </c>
+      <c r="L19" s="77" t="n">
+        <v>243</v>
+      </c>
+      <c r="M19" s="77" t="n">
+        <v>242</v>
+      </c>
+      <c r="N19" s="78" t="n">
+        <v>2812</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="76" t="inlineStr">
+        <is>
+          <t>MT/Premium</t>
+        </is>
+      </c>
+      <c r="B20" s="77" t="n">
+        <v>82</v>
+      </c>
+      <c r="C20" s="77" t="n">
+        <v>117</v>
+      </c>
+      <c r="D20" s="77" t="n">
+        <v>124</v>
+      </c>
+      <c r="E20" s="77" t="n">
+        <v>175</v>
+      </c>
+      <c r="F20" s="77" t="n">
+        <v>224</v>
+      </c>
+      <c r="G20" s="77" t="n">
+        <v>341</v>
+      </c>
+      <c r="H20" s="77" t="n">
+        <v>419</v>
+      </c>
+      <c r="I20" s="77" t="n">
+        <v>313</v>
+      </c>
+      <c r="J20" s="77" t="n">
+        <v>286</v>
+      </c>
+      <c r="K20" s="77" t="n">
+        <v>268</v>
+      </c>
+      <c r="L20" s="77" t="n">
+        <v>300</v>
+      </c>
+      <c r="M20" s="77" t="n">
+        <v>304</v>
+      </c>
+      <c r="N20" s="78" t="n">
+        <v>2953</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="76" t="inlineStr">
+        <is>
+          <t>MT/Group</t>
+        </is>
+      </c>
+      <c r="B21" s="77" t="n">
+        <v>89</v>
+      </c>
+      <c r="C21" s="77" t="n">
+        <v>100</v>
+      </c>
+      <c r="D21" s="77" t="n">
+        <v>83</v>
+      </c>
+      <c r="E21" s="77" t="n">
+        <v>144</v>
+      </c>
+      <c r="F21" s="77" t="n">
+        <v>148</v>
+      </c>
+      <c r="G21" s="77" t="n">
+        <v>200</v>
+      </c>
+      <c r="H21" s="77" t="n">
+        <v>248</v>
+      </c>
+      <c r="I21" s="77" t="n">
+        <v>205</v>
+      </c>
+      <c r="J21" s="77" t="n">
+        <v>198</v>
+      </c>
+      <c r="K21" s="77" t="n">
+        <v>184</v>
+      </c>
+      <c r="L21" s="77" t="n">
+        <v>207</v>
+      </c>
+      <c r="M21" s="77" t="n">
+        <v>219</v>
+      </c>
+      <c r="N21" s="78" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="63" t="inlineStr">
+        <is>
+          <t>TOTAL (all dims)</t>
+        </is>
+      </c>
+      <c r="B22" s="64" t="n">
+        <v>1573</v>
+      </c>
+      <c r="C22" s="64" t="n">
+        <v>1126</v>
+      </c>
+      <c r="D22" s="64" t="n">
+        <v>816</v>
+      </c>
+      <c r="E22" s="64" t="n">
+        <v>1319</v>
+      </c>
+      <c r="F22" s="64" t="n">
+        <v>1558</v>
+      </c>
+      <c r="G22" s="64" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H22" s="64" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I22" s="64" t="n">
+        <v>1466</v>
+      </c>
+      <c r="J22" s="64" t="n">
+        <v>1354</v>
+      </c>
+      <c r="K22" s="64" t="n">
+        <v>1284</v>
+      </c>
+      <c r="L22" s="64" t="n">
+        <v>1420</v>
+      </c>
+      <c r="M22" s="64" t="n">
+        <v>1449</v>
+      </c>
+      <c r="N22" s="64" t="n">
+        <v>17222</v>
+      </c>
+    </row>
+    <row r="23" ht="13" customHeight="1">
+      <c r="A23" s="79" t="inlineStr">
+        <is>
+          <t>PLAN input (for check)</t>
+        </is>
+      </c>
+      <c r="B23" s="80" t="n">
+        <v>1573</v>
+      </c>
+      <c r="C23" s="80" t="n">
+        <v>1127</v>
+      </c>
+      <c r="D23" s="80" t="n">
+        <v>816</v>
+      </c>
+      <c r="E23" s="80" t="n">
+        <v>1318</v>
+      </c>
+      <c r="F23" s="80" t="n">
+        <v>1557</v>
+      </c>
+      <c r="G23" s="80" t="n">
+        <v>2007</v>
+      </c>
+      <c r="H23" s="80" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I23" s="80" t="n">
+        <v>1467</v>
+      </c>
+      <c r="J23" s="80" t="n">
+        <v>1354</v>
+      </c>
+      <c r="K23" s="80" t="n">
+        <v>1284</v>
+      </c>
+      <c r="L23" s="80" t="n">
+        <v>1420</v>
+      </c>
+      <c r="M23" s="80" t="n">
+        <v>1450</v>
+      </c>
+      <c r="N23" s="80" t="n">
+        <v>17223</v>
+      </c>
+    </row>
+    <row r="24" ht="12" customHeight="1">
+      <c r="A24" s="79" t="inlineStr">
+        <is>
+          <t>diff (rounding)</t>
+        </is>
+      </c>
+      <c r="B24" s="81" t="n"/>
+      <c r="C24" s="81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="81" t="n"/>
+      <c r="H24" s="81" t="n"/>
+      <c r="I24" s="81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J24" s="81" t="n"/>
+      <c r="K24" s="81" t="n"/>
+      <c r="L24" s="81" t="n"/>
+      <c r="M24" s="81" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1147,7 +2503,7 @@
         <v>103</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>26</v>
+        <v>370</v>
       </c>
       <c r="H3" s="11" t="n">
         <v>221</v>
@@ -1193,7 +2549,7 @@
         <v>281</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>66</v>
+        <v>416</v>
       </c>
       <c r="H4" s="11" t="n">
         <v>486</v>
@@ -1239,7 +2595,7 @@
         <v>420</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>108</v>
+        <v>370</v>
       </c>
       <c r="H5" s="11" t="n">
         <v>744</v>
@@ -1285,7 +2641,7 @@
         <v>193</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>70</v>
+        <v>310</v>
       </c>
       <c r="H6" s="11" t="n">
         <v>155</v>
@@ -1331,7 +2687,7 @@
         <v>355</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>109</v>
+        <v>341</v>
       </c>
       <c r="H7" s="11" t="n">
         <v>181</v>
@@ -1377,7 +2733,7 @@
         <v>62</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>17</v>
+        <v>200</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>181</v>
@@ -1423,7 +2779,7 @@
         <v>1414</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>396</v>
+        <v>2007</v>
       </c>
       <c r="H9" s="14" t="n">
         <v>1968</v>
@@ -1476,7 +2832,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7565,7 +8921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15663,7 +17019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19052,7 +20408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19185,7 +20541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20028,7 +21384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20211,262 +21567,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>НАСТРОЙКИ МОДЕЛИ  —  меняй жёлтые ячейки, сохрани, перезапусти forecast_2026_v3.py</t>
-        </is>
-      </c>
-      <c r="B1" s="58" t="n"/>
-      <c r="C1" s="59" t="n"/>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Параметр</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
-          <t>Описание / Как влияет</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
-        <is>
-          <t>── ОКНО ДАННЫХ И ПРОГНОЗА ──</t>
-        </is>
-      </c>
-      <c r="B3" s="58" t="n"/>
-      <c r="C3" s="59" t="n"/>
-    </row>
-    <row r="4" ht="47" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>data_cutoff</t>
-        </is>
-      </c>
-      <c r="B4" s="56" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C4" s="30" t="inlineStr">
-        <is>
-          <t>Дата последних данных. Месяцы ДО этой даты используют режим data/blend. Например: 2024-12-31 = данные по декабрь 2024, прогноз с января 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>cal_window_start</t>
-        </is>
-      </c>
-      <c r="B5" s="56" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="C5" s="30" t="inlineStr">
-        <is>
-          <t>Начало окна калибровки рейтов/долей/AOV. Формат: YYYY-MM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="25" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>cal_window_end</t>
-        </is>
-      </c>
-      <c r="B6" s="56" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>Конец окна калибровки. По умолчанию — последний полный месяц до data_cutoff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="14" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>forecast_start</t>
-        </is>
-      </c>
-      <c r="B7" s="56" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="C7" s="30" t="inlineStr">
-        <is>
-          <t>Первый месяц прогноза. Формат: YYYY-MM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="29" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>forecast_end</t>
-        </is>
-      </c>
-      <c r="B8" s="56" t="inlineStr">
-        <is>
-          <t>2026-12</t>
-        </is>
-      </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>Последний месяц прогноза. Например: 2027-05 = прогноз на 12 мес. вперёд от data_cutoff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="41" t="inlineStr">
-        <is>
-          <t>── КОРРЕКЦИЯ AOV ──</t>
-        </is>
-      </c>
-      <c r="B9" s="58" t="n"/>
-      <c r="C9" s="59" t="n"/>
-    </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>aov_adjustment_factor</t>
-        </is>
-      </c>
-      <c r="B10" s="57" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="30" t="inlineStr">
-        <is>
-          <t>❗ ПОЧЕМУ AOV может отличаться от факта:
-1. Цены calibrated на среднем (mean) — чувствительно к выбросам и сезонности.
-2. Пакеты pkg=999 (кастомные) исключены из калибровки — реальный AOV выше.
-3. Распределение пакетов июл-дек 2025 может отличаться от 2026.
-→ Коэффициент 1.10 = скорректировать выручку на 10% (бэктест: Jan 2026 = -0.2%).
-→ Поставь 1.0 чтобы без коррекции. Меняй под обновлённые данные.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>── РОСТ ЦЕН ──</t>
-        </is>
-      </c>
-      <c r="B11" s="58" t="n"/>
-      <c r="C11" s="59" t="n"/>
-    </row>
-    <row r="12" ht="21" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>price_growth_pct_per_quarter</t>
-        </is>
-      </c>
-      <c r="B12" s="57" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>Рост цены за урок в квартал (3% = +3%/квартал). База = Q3 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="14" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>price_base_year</t>
-        </is>
-      </c>
-      <c r="B13" s="56" t="n">
-        <v>2025</v>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>Год базового периода для роста цен.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="43" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>price_base_quarter</t>
-        </is>
-      </c>
-      <c r="B14" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>Квартал базового периода (4 = Q4 = окт-дек, рекомендуется). Диагностика: Q3→Q4 рост +15%, поэтому Q4 = более точная база для 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="41" t="inlineStr">
-        <is>
-          <t>── КОРРЕКТИРОВКА RETENTION ──</t>
-        </is>
-      </c>
-      <c r="B15" s="58" t="n"/>
-      <c r="C15" s="59" t="n"/>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>retention_adjustment</t>
-        </is>
-      </c>
-      <c r="B16" s="57" t="n">
-        <v>1</v>
-      </c>
-      <c r="C16" s="30" t="inlineStr">
-        <is>
-          <t>❗ ТРЕНД СНИЖЕНИЯ RETENTION:
-May 2026 actual: retention=38.4% vs калибровка Jul-Dec 2025: 43.6% (-12%).
-Retention постепенно снижается год к году.
-→ 0.88 = умножить все retention[pno] на 0.88 (-12%)
-→ 1.0  = без коррекции (использовать 2025 ставки)
-Рекомендация для 2026 прогноза: попробуй 0.88-0.92.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A15:C15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>